<commit_message>
fix: dedupe IT and Pharma companies (Manufacturing already clean)
Removed 3 duplicate entries sharing a website with another row: SAP
America, Inc. (kept SAP, IT), Illumina Ventures (kept Illumina, Inc. -
the VC arm isn't a training prospect, Pharma), Incyte Genomics, Inc.
(kept Incyte Corporation, its legacy name, Pharma). Manufacturing had
zero duplicates. Removed the same rows from the source xlsx files.

All 5 industries now confirmed duplicate-free by website hostname.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/PMP_IT_Companies_USA.xlsx
+++ b/research/PMP_IT_Companies_USA.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,12 +471,12 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>https://www.apple.com</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/320193/000032019325000079/aapl-20250927.htm</t>
         </is>
@@ -503,12 +503,12 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>https://www.microsoft.com</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/789019/000095017025100235/msft-20250630.htm</t>
         </is>
@@ -535,12 +535,12 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>https://www.abc.xyz</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1652044/000165204426000018/goog-20251231.htm</t>
         </is>
@@ -567,12 +567,12 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>https://www.amazon.com</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1018724/000101872426000004/amzn-20251231.htm</t>
         </is>
@@ -599,12 +599,12 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>https://about.meta.com</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1326801/000162828026003942/meta-20251231.htm</t>
         </is>
@@ -631,12 +631,12 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>https://www.intel.com</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/50863/000005086326000011/intc-20251227.htm</t>
         </is>
@@ -663,12 +663,12 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>https://www.cisco.com</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/858877/000085887725000111/csco-20250726.htm</t>
         </is>
@@ -695,12 +695,12 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>https://www.ibm.com</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/51143/000005114326000010/ibm-20251231.htm</t>
         </is>
@@ -727,12 +727,12 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>https://www.oracle.com</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1341439/000119312526277521/orcl-20260531.htm</t>
         </is>
@@ -751,7 +751,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SAP America, Inc.</t>
+          <t>Salesforce.com, Inc.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -759,26 +759,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sap.com</t>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.salesforce.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1108524/000110852426000060/crm-20260131.htm</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SAP Learning Hub is a company-wide digital platform delivering guided, expert-led, and hands-on upskilling across the SAP software portfolio | Integrated learning experience in SAP SuccessFactors combines mandatory compliance training with role-based and self-directed content, delivered partly through a Skillsoft content partnership | In 2025, SAP's learning organization partnered with Accenture to deliver personalized upskilling/reskilling training services from the C-suite to technical teams</t>
+          <t>Offers premium AI courses and certifications free via Trailhead learning platform through end of 2025 | Employees and external learners earned 2.6M+ AI and data badges on Trailhead since June 2023 | Runs Career Connect internal talent marketplace with AI career-coach agent recommending Trailhead content; 2025 goal to get 80% of ~76,453 employees fundamental AI skills</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SAP.com SuccessFactors Learning Hub pages; SAP news release on Accenture partnership</t>
+          <t>Salesforce FY2025 10-K human capital section, Salesforce newsroom</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Salesforce.com, Inc.</t>
+          <t>Dell Technologies Inc.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -786,31 +791,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>https://www.salesforce.com</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1108524/000110852426000060/crm-20260131.htm</t>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://www.dell.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1571996/000157199626000008/dell-20260130.htm</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Offers premium AI courses and certifications free via Trailhead learning platform through end of 2025 | Employees and external learners earned 2.6M+ AI and data badges on Trailhead since June 2023 | Runs Career Connect internal talent marketplace with AI career-coach agent recommending Trailhead content; 2025 goal to get 80% of ~76,453 employees fundamental AI skills</t>
+          <t>~108,000 employees (FY2025 10-K) with human capital section citing ongoing training and development offerings as part of talent strategy | Runs 'Dell Learning' portal (learning.dell.com) offering upskilling and vendor/technical certification pathways for employees and customers | Featured leadership development strategy built around structured internal education programs</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Salesforce FY2025 10-K human capital section, Salesforce newsroom</t>
+          <t>Dell Technologies FY2025 10-K (SEC), Dell Learning site</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dell Technologies Inc.</t>
+          <t>Hewlett Packard Enterprise Company</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -818,31 +823,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
-        <is>
-          <t>https://www.dell.com</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1571996/000157199626000008/dell-20260130.htm</t>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.hpe.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1645590/000164559025000130/hpe-20251031.htm</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>~108,000 employees (FY2025 10-K) with human capital section citing ongoing training and development offerings as part of talent strategy | Runs 'Dell Learning' portal (learning.dell.com) offering upskilling and vendor/technical certification pathways for employees and customers | Featured leadership development strategy built around structured internal education programs</t>
+          <t>HPE runs internal learning/organizational-development functions (dedicated Chief Learning Officer role) parallel to its customer-facing HPE Education Services training business | offers structured onboarding and technical upskilling paths given HPE Education Services' 35+ years leading IT/digital skills training | supports professional certification paths internally mirroring its external certification programs (e.g., HPE ATP/ASE)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Dell Technologies FY2025 10-K (SEC), Dell Learning site</t>
+          <t>HPE careers site, HPE Education Services marketing pages â€” no specific internal L&amp;D numbers found in filings</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Hewlett Packard Enterprise Company</t>
+          <t>HP Inc.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -850,31 +855,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>https://www.hpe.com</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1645590/000164559025000130/hpe-20251031.htm</t>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.hp.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/47217/000004721725000071/hpq-20251031.htm</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>HPE runs internal learning/organizational-development functions (dedicated Chief Learning Officer role) parallel to its customer-facing HPE Education Services training business | offers structured onboarding and technical upskilling paths given HPE Education Services' 35+ years leading IT/digital skills training | supports professional certification paths internally mirroring its external certification programs (e.g., HPE ATP/ASE)</t>
+          <t>~58,000 employees across 59 countries (FY2024/2025 10-K human capital section) with stated focus on continuous learning and development | Offers enterprise-wide skill development in software development, AI, data science, product management, communications, and strategic thinking | Extensive internal/external development program portfolio including targeted training for new people managers on coaching and inclusion</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>HPE careers site, HPE Education Services marketing pages â€” no specific internal L&amp;D numbers found in filings</t>
+          <t>HP Inc. FY2024/2025 10-K (SEC) human capital disclosures</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HP Inc.</t>
+          <t>VMware, Inc.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -882,31 +887,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>https://www.hp.com</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/47217/000004721725000071/hpq-20251031.htm</t>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.vmware.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=VMW</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>~58,000 employees across 59 countries (FY2024/2025 10-K human capital section) with stated focus on continuous learning and development | Offers enterprise-wide skill development in software development, AI, data science, product management, communications, and strategic thinking | Extensive internal/external development program portfolio including targeted training for new people managers on coaching and inclusion</t>
+          <t>VMware (now part of Broadcom since Nov 2023) offers 'VCF Learning' with role-based, on-demand and instructor-led training on VMware Cloud Foundation technologies via Learning@Broadcom portal | Provides formal VMware/VCF certification tracks (e.g., VCF Certified Professional) as career upskilling/reskilling pathways | Runs a VMware Cloud Foundation Certified Instructor Program to train and certify instructors delivering VMware technical education</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>HP Inc. FY2024/2025 10-K (SEC) human capital disclosures</t>
+          <t>Broadcom Support/Education (VMware) pages â€” no longer an independent SEC filer post-acquisition</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>VMware, Inc.</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -914,31 +919,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
-        <is>
-          <t>https://www.vmware.com</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=VMW</t>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.nvidia.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1045810/000104581026000021/nvda-20260125.htm</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>VMware (now part of Broadcom since Nov 2023) offers 'VCF Learning' with role-based, on-demand and instructor-led training on VMware Cloud Foundation technologies via Learning@Broadcom portal | Provides formal VMware/VCF certification tracks (e.g., VCF Certified Professional) as career upskilling/reskilling pathways | Runs a VMware Cloud Foundation Certified Instructor Program to train and certify instructors delivering VMware technical education</t>
+          <t>Offers on-the-job training courses and tuition reimbursement programs to subsidize educational programs and advanced certifications | Encourages internal job mobility as part of career-development philosophy ('build careers over their lifetime') | FY2026 employee turnover of 3.7%, well below the 16-17% semiconductor industry average, reflecting retention-focused development investment</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Broadcom Support/Education (VMware) pages â€” no longer an independent SEC filer post-acquisition</t>
+          <t>NVIDIA FY2026 10-K (SEC) Human Capital section</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NVIDIA Corporation</t>
+          <t>Advanced Micro Devices, Inc.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -946,31 +951,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>https://www.nvidia.com</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1045810/000104581026000021/nvda-20260125.htm</t>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.amd.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/2488/000000248826000018/amd-20251227.htm</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Offers on-the-job training courses and tuition reimbursement programs to subsidize educational programs and advanced certifications | Encourages internal job mobility as part of career-development philosophy ('build careers over their lifetime') | FY2026 employee turnover of 3.7%, well below the 16-17% semiconductor industry average, reflecting retention-focused development investment</t>
+          <t>Provides tuition reimbursement for eligible employees to pursue university education or achieve advanced professional certifications | Runs manager and leadership development programs described as highly rated, with majority of new leaders promoted from within | Operates an enterprise-wide mentoring program pairing employees with experienced colleagues for skills development and onboarding support</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>NVIDIA FY2026 10-K (SEC) Human Capital section</t>
+          <t>AMD FY2025 10-K (SEC) Human Capital section</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices, Inc.</t>
+          <t>Texas Instruments Incorporated</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -978,31 +983,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
-        <is>
-          <t>https://www.amd.com</t>
-        </is>
-      </c>
-      <c r="D18" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/2488/000000248826000018/amd-20251227.htm</t>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.ti.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/97476/000009747626000059/txn-20251231.htm</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Provides tuition reimbursement for eligible employees to pursue university education or achieve advanced professional certifications | Runs manager and leadership development programs described as highly rated, with majority of new leaders promoted from within | Operates an enterprise-wide mentoring program pairing employees with experienced colleagues for skills development and onboarding support</t>
+          <t>Tuition Reimbursement Program covers 50% of costs for college degrees or job-relevant coursework | 'Make an Impact' is a one-year structured development program for new college graduates combining hands-on experience, training, and professional courses | Offers internal rotation programs letting employees work across different teams and learn from technical experts</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AMD FY2025 10-K (SEC) Human Capital section</t>
+          <t>TI careers/investor site and Educational Assistance Program portal</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Texas Instruments Incorporated</t>
+          <t>Broadcom Inc.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1010,31 +1015,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
-        <is>
-          <t>https://www.ti.com</t>
-        </is>
-      </c>
-      <c r="D19" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/97476/000009747626000059/txn-20251231.htm</t>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://www.broadcom.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1730168/000173016825000121/avgo-20251102.htm</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Tuition Reimbursement Program covers 50% of costs for college degrees or job-relevant coursework | 'Make an Impact' is a one-year structured development program for new college graduates combining hands-on experience, training, and professional courses | Offers internal rotation programs letting employees work across different teams and learn from technical experts</t>
+          <t>Requires all employees and contractors to complete training on Code of Ethics, harassment prevention, cybersecurity/data privacy, human rights, and anti-corruption | Reimbursed approximately $540,000 in tuition expenses in FY2025 through its Educational Assistance Program covering academic classes and degree programs | Recognized by Newsweek in 2025 as one of America's Greatest Workplaces, citing training and career progression</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TI careers/investor site and Educational Assistance Program portal</t>
+          <t>Broadcom FY2025 10-K (SEC) Human Capital / Workforce section</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Broadcom Inc.</t>
+          <t>Micron Technology, Inc.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1042,31 +1047,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>https://www.broadcom.com</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1730168/000173016825000121/avgo-20251102.htm</t>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://www.micron.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/723125/000072312525000028/mu-20250828.htm</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Requires all employees and contractors to complete training on Code of Ethics, harassment prevention, cybersecurity/data privacy, human rights, and anti-corruption | Reimbursed approximately $540,000 in tuition expenses in FY2025 through its Educational Assistance Program covering academic classes and degree programs | Recognized by Newsweek in 2025 as one of America's Greatest Workplaces, citing training and career progression</t>
+          <t>Micron University is a self-directed online learning platform built with world-class learning-solution partners for skills-based employee growth | Leadership development ecosystem ('Micron Leadership Accelerated') supports transitions from new leader to executive roles | Registered Apprenticeship Program combines paid on-the-job training with Micron-covered tuition under an 'earn and learn' model for aspiring technicians</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Broadcom FY2025 10-K (SEC) Human Capital / Workforce section</t>
+          <t>Micron investor news release and careers/apprenticeship pages</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Micron Technology, Inc.</t>
+          <t>Western Digital Corporation</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1074,31 +1079,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
-        <is>
-          <t>https://www.micron.com</t>
-        </is>
-      </c>
-      <c r="D21" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/723125/000072312525000028/mu-20250828.htm</t>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://www.westerndigital.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/106040/000010604025000038/wdc-20250627.htm</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Micron University is a self-directed online learning platform built with world-class learning-solution partners for skills-based employee growth | Leadership development ecosystem ('Micron Leadership Accelerated') supports transitions from new leader to executive roles | Registered Apprenticeship Program combines paid on-the-job training with Micron-covered tuition under an 'earn and learn' model for aspiring technicians</t>
+          <t>offers structured onboarding and role-specific technical/engineering training given large global manufacturing workforce | provides leadership development programs for managers as part of standard tech-industry HR practice | 10-K human capital section references training/retention programs but does not disclose specific hours or dollar figures</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Micron investor news release and careers/apprenticeship pages</t>
+          <t>WDC FY2025 10-K (SEC) human capital section â€” no specific training metrics found</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Western Digital Corporation</t>
+          <t>Seagate Technology Holdings plc</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1106,31 +1111,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
-        <is>
-          <t>https://www.westerndigital.com</t>
-        </is>
-      </c>
-      <c r="D22" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/106040/000010604025000038/wdc-20250627.htm</t>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://www.seagate.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1137789/000113778925000157/stx-20250627.htm</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>offers structured onboarding and role-specific technical/engineering training given large global manufacturing workforce | provides leadership development programs for managers as part of standard tech-industry HR practice | 10-K human capital section references training/retention programs but does not disclose specific hours or dollar figures</t>
+          <t>Employees completed over 2.5 million learning hours in a recent fiscal year (per Seagate ESG/Sustainability Performance Report) | Training portfolio includes mentoring/coaching, e-learning, LinkedIn Learning classroom training, and on-the-job training covering leadership, technical skills, health/safety, and environment | FY2025 Sustainability Report names 'Training and Skills Development' as a formal material ESG topic</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>WDC FY2025 10-K (SEC) human capital section â€” no specific training metrics found</t>
+          <t>Seagate FY2025 Sustainability Report</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Seagate Technology Holdings plc</t>
+          <t>Qualcomm Incorporated</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1138,31 +1143,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
-        <is>
-          <t>https://www.seagate.com</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1137789/000113778925000157/stx-20250627.htm</t>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://www.qualcomm.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/804328/000080432825000085/qcom-20250928.htm</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Employees completed over 2.5 million learning hours in a recent fiscal year (per Seagate ESG/Sustainability Performance Report) | Training portfolio includes mentoring/coaching, e-learning, LinkedIn Learning classroom training, and on-the-job training covering leadership, technical skills, health/safety, and environment | FY2025 Sustainability Report names 'Training and Skills Development' as a formal material ESG topic</t>
+          <t>Employees accessed over 110,000 hours of technical training in 2025, plus leadership development, coaching, and generative AI learning opportunities | Offers the Accelerate program for first-time managers/new leaders and Mentoring Matters, a structured mentor-mentee eLearning program | Provides tuition reimbursement alongside engineering and professional-skills development tracks</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Seagate FY2025 Sustainability Report</t>
+          <t>Qualcomm 2025 Corporate Responsibility Report</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Qualcomm Incorporated</t>
+          <t>Palantir Technologies Inc.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1170,31 +1175,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
-        <is>
-          <t>https://www.qualcomm.com</t>
-        </is>
-      </c>
-      <c r="D24" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/804328/000080432825000085/qcom-20250928.htm</t>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://www.palantir.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1321655/000132165526000011/pltr-20251231.htm</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Employees accessed over 110,000 hours of technical training in 2025, plus leadership development, coaching, and generative AI learning opportunities | Offers the Accelerate program for first-time managers/new leaders and Mentoring Matters, a structured mentor-mentee eLearning program | Provides tuition reimbursement alongside engineering and professional-skills development tracks</t>
+          <t>relies heavily on internal, hands-on 'forward-deployed engineer' style training rather than formal named academies, typical of Palantir's engineering-led culture | invests in onboarding and continuous technical upskilling given deep product complexity (Foundry, AIP), but doesn't disclose training hours/spend | 10-K human capital section states objectives include 'recruiting, retaining, training, and motivating personnel' without specific metrics; runs a public 'Palantir Learn' training portal for platform certification</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Qualcomm 2025 Corporate Responsibility Report</t>
+          <t>Palantir FY2024/2025 10-K (SEC) human capital section; learn.palantir.com</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Palantir Technologies Inc.</t>
+          <t>Zoom Video Communications, Inc.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1202,31 +1207,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
-        <is>
-          <t>https://www.palantir.com</t>
-        </is>
-      </c>
-      <c r="D25" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1321655/000132165526000011/pltr-20251231.htm</t>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://www.zoom.us</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1585521/000158552126000030/zm-20260131.htm</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>relies heavily on internal, hands-on 'forward-deployed engineer' style training rather than formal named academies, typical of Palantir's engineering-led culture | invests in onboarding and continuous technical upskilling given deep product complexity (Foundry, AIP), but doesn't disclose training hours/spend | 10-K human capital section states objectives include 'recruiting, retaining, training, and motivating personnel' without specific metrics; runs a public 'Palantir Learn' training portal for platform certification</t>
+          <t>offers professional development stipends/reimbursement rather than large-scale named leadership academies | given 'deliver happiness' culture, invests in internal learning platform (employee-learning.zoom.us) for product and skills training | 10-K human capital disclosures focus on culture/DEI rather than disclosing specific training hours or L&amp;D spend</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Palantir FY2024/2025 10-K (SEC) human capital section; learn.palantir.com</t>
+          <t>Zoom 10-K human capital sections; employee-learning.zoom.us</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Zoom Video Communications, Inc.</t>
+          <t>Twilio Inc.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1234,31 +1239,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
-        <is>
-          <t>https://www.zoom.us</t>
-        </is>
-      </c>
-      <c r="D26" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1585521/000158552126000030/zm-20260131.htm</t>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://www.twilio.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1447669/000144766926000021/twlo-20251231.htm</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>offers professional development stipends/reimbursement rather than large-scale named leadership academies | given 'deliver happiness' culture, invests in internal learning platform (employee-learning.zoom.us) for product and skills training | 10-K human capital disclosures focus on culture/DEI rather than disclosing specific training hours or L&amp;D spend</t>
+          <t>Twilio's Compensation and Talent Management Committee oversees human capital activities including talent management and development company-wide | Offers employees a $30/month book/learning stipend plus professional coaching through Bravely | 'Twilio Recharge' gives employees a paid 4-week sabbatical after every 3 years of service, reinforcing long-term career investment</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Zoom 10-K human capital sections; employee-learning.zoom.us</t>
+          <t>Twilio FY2025 10-K (SEC)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Twilio Inc.</t>
+          <t>Dropbox, Inc.</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1266,31 +1271,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>https://www.twilio.com</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1447669/000144766926000021/twlo-20251231.htm</t>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1467623/000146762326000008/dbx-20251231.htm</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Twilio's Compensation and Talent Management Committee oversees human capital activities including talent management and development company-wide | Offers employees a $30/month book/learning stipend plus professional coaching through Bravely | 'Twilio Recharge' gives employees a paid 4-week sabbatical after every 3 years of service, reinforcing long-term career investment</t>
+          <t>Launched an internal 'AI Academy' in 2025 with multiple tracks to upskill employees on responsible and effective AI use | Offers tuition reimbursement plus a continuing education stipend, mentorship programs, and structured leadership development courses | Uses 'coaching pods,' stretch projects, and digital learning paths as part of its Virtual First career-development ecosystem</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Twilio FY2025 10-K (SEC)</t>
+          <t>Dropbox FY2025 10-K/ARS; Dropbox Blog</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dropbox, Inc.</t>
+          <t>Atlassian Corporation Plc</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1298,31 +1303,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1467623/000146762326000008/dbx-20251231.htm</t>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://www.atlassian.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1650372/000165037225000036/team-20250630.htm</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Launched an internal 'AI Academy' in 2025 with multiple tracks to upskill employees on responsible and effective AI use | Offers tuition reimbursement plus a continuing education stipend, mentorship programs, and structured leadership development courses | Uses 'coaching pods,' stretch projects, and digital learning paths as part of its Virtual First career-development ecosystem</t>
+          <t>Provides employees a dedicated learning/tuition budget alongside 'Atlassian University' for structured on-demand courses, learning paths, and certifications | Runs specialized upskilling programs including an internal 'AI School' and ML reading groups | Quarterly 'ShipIt' hackathons let staff form cross-functional teams to build and pitch new ideas outside their day jobs</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Dropbox FY2025 10-K/ARS; Dropbox Blog</t>
+          <t>Atlassian FY2025 10-K (SEC)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Atlassian Corporation Plc</t>
+          <t>DocuSign, Inc.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1330,31 +1335,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
-        <is>
-          <t>https://www.atlassian.com</t>
-        </is>
-      </c>
-      <c r="D29" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1650372/000165037225000036/team-20250630.htm</t>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://www.docusign.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1261333/000126133326000021/docu-20260131.htm</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Provides employees a dedicated learning/tuition budget alongside 'Atlassian University' for structured on-demand courses, learning paths, and certifications | Runs specialized upskilling programs including an internal 'AI School' and ML reading groups | Quarterly 'ShipIt' hackathons let staff form cross-functional teams to build and pitch new ideas outside their day jobs</t>
+          <t>Offers Education Assistance/tuition reimbursement of $5,000 per employee per year, usable beyond degree programs for relevant training and certs | 'DocuSign University' provides role-based learning paths with industry-recognized technical certification options | Combines in-person and online Learning &amp; Development training as a core part of its employee value proposition</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Atlassian FY2025 10-K (SEC)</t>
+          <t>DocuSign careers/benefits pages; DocuSign University site</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DocuSign, Inc.</t>
+          <t>CrowdStrike Holdings, Inc.</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1362,31 +1367,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
-        <is>
-          <t>https://www.docusign.com</t>
-        </is>
-      </c>
-      <c r="D30" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1261333/000126133326000021/docu-20260131.htm</t>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://www.crowdstrike.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1535527/000153552726000010/crwd-20260131.htm</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Offers Education Assistance/tuition reimbursement of $5,000 per employee per year, usable beyond degree programs for relevant training and certs | 'DocuSign University' provides role-based learning paths with industry-recognized technical certification options | Combines in-person and online Learning &amp; Development training as a core part of its employee value proposition</t>
+          <t>10-K states CrowdStrike 'invests in CrowdStrikers' career growth through comprehensive learning and development programs at all levels, from intern to executive' | Internal training includes employee resource group programming and allyship training as part of its D&amp;I learning initiatives | Runs 'CrowdStrike University,' a large-scale certification/LMS platform primarily for customers/partners, reflecting the company's broader certification-driven training culture</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>DocuSign careers/benefits pages; DocuSign University site</t>
+          <t>CrowdStrike FY2026 10-K (SEC); CrowdStrike University site</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CrowdStrike Holdings, Inc.</t>
+          <t>Okta, Inc.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1394,31 +1399,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
-        <is>
-          <t>https://www.crowdstrike.com</t>
-        </is>
-      </c>
-      <c r="D31" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1535527/000153552726000010/crwd-20260131.htm</t>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://www.okta.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1660134/000166013426000020/okta-20260131.htm</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>10-K states CrowdStrike 'invests in CrowdStrikers' career growth through comprehensive learning and development programs at all levels, from intern to executive' | Internal training includes employee resource group programming and allyship training as part of its D&amp;I learning initiatives | Runs 'CrowdStrike University,' a large-scale certification/LMS platform primarily for customers/partners, reflecting the company's broader certification-driven training culture</t>
+          <t>Runs formal employee onboarding program plus a dedicated manager development program for people managers | Offers technical training program specifically for new technical hires on Okta's product offerings | Provides blended learning mix: in-person, virtual, social/self-directed learning, mentoring, coaching and external development</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>CrowdStrike FY2026 10-K (SEC); CrowdStrike University site</t>
+          <t>Okta FY2026 10-K (SEC) human capital section</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Okta, Inc.</t>
+          <t>Snowflake Inc.</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1426,31 +1431,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
-        <is>
-          <t>https://www.okta.com</t>
-        </is>
-      </c>
-      <c r="D32" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1660134/000166013426000020/okta-20260131.htm</t>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://www.snowflake.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1640147/000164014726000008/snow-20260131.htm</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Runs formal employee onboarding program plus a dedicated manager development program for people managers | Offers technical training program specifically for new technical hires on Okta's product offerings | Provides blended learning mix: in-person, virtual, social/self-directed learning, mentoring, coaching and external development</t>
+          <t>maintains structured onboarding and role-based technical/product training given its rapid engineering headcount growth | requires all employees to complete annual ethics/compliance certification tied to a broader compliance training program | offers internal learning stipends or manager development tracks typical of high-growth SaaS peers, though no specific $ or hours figure is disclosed publicly</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Okta FY2026 10-K (SEC) human capital section</t>
+          <t>Snowflake ESG page â€” no quantified L&amp;D figures found</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Snowflake Inc.</t>
+          <t>Datadog, Inc.</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1458,31 +1463,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C33" s="1" t="inlineStr">
-        <is>
-          <t>https://www.snowflake.com</t>
-        </is>
-      </c>
-      <c r="D33" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1640147/000164014726000008/snow-20260131.htm</t>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.datadoghq.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1561550/000162828026008819/ddog-20251231.htm</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>maintains structured onboarding and role-based technical/product training given its rapid engineering headcount growth | requires all employees to complete annual ethics/compliance certification tied to a broader compliance training program | offers internal learning stipends or manager development tracks typical of high-growth SaaS peers, though no specific $ or hours figure is disclosed publicly</t>
+          <t>Runs a biannual company-wide 'Learning Week' for employee-to-employee knowledge sharing | Provides employees access to 3,500+ business, technical, and personal-development e-learning courses via licensed platforms | Operates a day-one mentorship program plus an internal 'embed' program letting staff shadow other teams; about 1 in 3 employees move internally each year</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Snowflake ESG page â€” no quantified L&amp;D figures found</t>
+          <t>Datadog Careers - Learning &amp; Development page</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Datadog, Inc.</t>
+          <t>Cloudflare, Inc.</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1490,31 +1495,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C34" s="1" t="inlineStr">
-        <is>
-          <t>https://www.datadoghq.com</t>
-        </is>
-      </c>
-      <c r="D34" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1561550/000162828026008819/ddog-20251231.htm</t>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://www.cloudflare.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1477333/000147733326000016/cloud-20251231.htm</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Runs a biannual company-wide 'Learning Week' for employee-to-employee knowledge sharing | Provides employees access to 3,500+ business, technical, and personal-development e-learning courses via licensed platforms | Operates a day-one mentorship program plus an internal 'embed' program letting staff shadow other teams; about 1 in 3 employees move internally each year</t>
+          <t>Operates 'Cloudflare University' to deliver structured product/technical training to employees (also extended to partners and customers) | Backs a public Learning Center with self-study and instructor-led cybersecurity/network training content used for internal upskilling | Supports role-based Cloudflare Certified Specialist (CCS) certification tracks relevant to technical staff development</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Datadog Careers - Learning &amp; Development page</t>
+          <t>Cloudflare.com Learning Center / Trust Hub certification pages</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cloudflare, Inc.</t>
+          <t>HubSpot, Inc.</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1522,31 +1527,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C35" s="1" t="inlineStr">
-        <is>
-          <t>https://www.cloudflare.com</t>
-        </is>
-      </c>
-      <c r="D35" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1477333/000147733326000016/cloud-20251231.htm</t>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.hubspot.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1404655/000119312526046646/hubs-20251231.htm</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Operates 'Cloudflare University' to deliver structured product/technical training to employees (also extended to partners and customers) | Backs a public Learning Center with self-study and instructor-led cybersecurity/network training content used for internal upskilling | Supports role-based Cloudflare Certified Specialist (CCS) certification tracks relevant to technical staff development</t>
+          <t>Offers up to $5,000 per employee per year in tuition reimbursement for university courses, workshops, or online classes | Runs 'Learn@HubSpot,' an internal video-based L&amp;D platform connecting employee teachers and learners company-wide | Culture built around 'Always Be Growing' motto, including dedicated manager-training classes and a free-book program for professional development</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Cloudflare.com Learning Center / Trust Hub certification pages</t>
+          <t>HubSpot Culture Code / Eden Workplace blog</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>HubSpot, Inc.</t>
+          <t>New Relic, Inc.</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1554,31 +1559,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C36" s="1" t="inlineStr">
-        <is>
-          <t>https://www.hubspot.com</t>
-        </is>
-      </c>
-      <c r="D36" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1404655/000119312526046646/hubs-20251231.htm</t>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://www.newrelic.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=NEWR</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Offers up to $5,000 per employee per year in tuition reimbursement for university courses, workshops, or online classes | Runs 'Learn@HubSpot,' an internal video-based L&amp;D platform connecting employee teachers and learners company-wide | Culture built around 'Always Be Growing' motto, including dedicated manager-training classes and a free-book program for professional development</t>
+          <t>New Relic ran an onboarding, coaching, and mentoring program for new hires, with structured career-planning resources for skill growth | offered a Tuition Reimbursement Program covering roughly 50% of costs for job-relevant college degrees or courses | provided leadership-track seminars and courses (via New Relic University) aimed at developing employees into people-management roles</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>HubSpot Culture Code / Eden Workplace blog</t>
+          <t>Levels.fyi/Glassdoor benefit summaries; New Relic University site â€” company taken private 2023</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>New Relic, Inc.</t>
+          <t>Splunk Inc.</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1586,31 +1591,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C37" s="1" t="inlineStr">
-        <is>
-          <t>https://www.newrelic.com</t>
-        </is>
-      </c>
-      <c r="D37" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=NEWR</t>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://www.splunk.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=SPLK</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>New Relic ran an onboarding, coaching, and mentoring program for new hires, with structured career-planning resources for skill growth | offered a Tuition Reimbursement Program covering roughly 50% of costs for job-relevant college degrees or courses | provided leadership-track seminars and courses (via New Relic University) aimed at developing employees into people-management roles</t>
+          <t>Pre-acquisition, Splunk invested in leadership and learning programs combining live courses, mentor programs, technical/product/sales training, and manager-led development across the company | Splunk Academic Alliance partnered with colleges/universities on data and security training curriculum, later integrated into Cisco's Networking Academy | Since Cisco completed the March 2024 acquisition, Splunk's training programs have been folded into Cisco's broader learning ecosystem</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Levels.fyi/Glassdoor benefit summaries; New Relic University site â€” company taken private 2023</t>
+          <t>Splunk pre-acquisition proxy/culture statements; Cisco/Splunk blog posts on Academic Alliance integration</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Splunk Inc.</t>
+          <t>ServiceNow, Inc.</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1618,31 +1623,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C38" s="1" t="inlineStr">
-        <is>
-          <t>https://www.splunk.com</t>
-        </is>
-      </c>
-      <c r="D38" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=SPLK</t>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://www.servicenow.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1373715/000137371526000007/now-20251231.htm</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Pre-acquisition, Splunk invested in leadership and learning programs combining live courses, mentor programs, technical/product/sales training, and manager-led development across the company | Splunk Academic Alliance partnered with colleges/universities on data and security training curriculum, later integrated into Cisco's Networking Academy | Since Cisco completed the March 2024 acquisition, Splunk's training programs have been folded into Cisco's broader learning ecosystem</t>
+          <t>In 2025 ServiceNow launched ServiceNow University, a free AI-powered learning hub open to employees, customers and partners, targeting 3 million learners trained by end of 2027 | Offers 600+ free courses and 18 job-related certification paths combining instructor-led training, on-demand learning, and real-world practical experience | RiseUp with ServiceNow upskills people without traditional tech backgrounds into ServiceNow ecosystem careers, feeding ServiceNow's own hiring and partner/customer certification pipeline</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Splunk pre-acquisition proxy/culture statements; Cisco/Splunk blog posts on Academic Alliance integration</t>
+          <t>ServiceNow University/RiseUp press coverage; servicenow.com/university</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ServiceNow, Inc.</t>
+          <t>Workday, Inc.</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1650,31 +1655,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C39" s="1" t="inlineStr">
-        <is>
-          <t>https://www.servicenow.com</t>
-        </is>
-      </c>
-      <c r="D39" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1373715/000137371526000007/now-20251231.htm</t>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://www.workday.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1327811/000132781126000014/wday-20260131.htm</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>In 2025 ServiceNow launched ServiceNow University, a free AI-powered learning hub open to employees, customers and partners, targeting 3 million learners trained by end of 2027 | Offers 600+ free courses and 18 job-related certification paths combining instructor-led training, on-demand learning, and real-world practical experience | RiseUp with ServiceNow upskills people without traditional tech backgrounds into ServiceNow ecosystem careers, feeding ServiceNow's own hiring and partner/customer certification pipeline</t>
+          <t>provides employees instant access to third-party learning platforms/content libraries plus internal development resources as part of its human capital program | built 'Career Hub,' an AI-driven internal tool that recommends skill-building content and internal job opportunities to employees, reflecting Workday's own HCM/Skills Cloud technology applied internally | emphasizes internal mobility and career/development planning for employees as part of its 10-K human capital disclosures, though no specific training-hour or dollar figures are publicly broken out</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>ServiceNow University/RiseUp press coverage; servicenow.com/university</t>
+          <t>Workday 10-K human capital section summaries; workday.com Career Hub pages</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Workday, Inc.</t>
+          <t>Autodesk, Inc.</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1682,31 +1687,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C40" s="1" t="inlineStr">
-        <is>
-          <t>https://www.workday.com</t>
-        </is>
-      </c>
-      <c r="D40" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327811/000132781126000014/wday-20260131.htm</t>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.autodesk.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/769397/000076939726000015/adsk-20260131.htm</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>provides employees instant access to third-party learning platforms/content libraries plus internal development resources as part of its human capital program | built 'Career Hub,' an AI-driven internal tool that recommends skill-building content and internal job opportunities to employees, reflecting Workday's own HCM/Skills Cloud technology applied internally | emphasizes internal mobility and career/development planning for employees as part of its 10-K human capital disclosures, though no specific training-hour or dollar figures are publicly broken out</t>
+          <t>Ran a six-month Tech Lead Development Program (TLDP) cohort for rising non-technical leaders, with 66% of participants promoted or given new responsibilities during/after the program and 88% saying it helped drive success for their organization | Runs 'NEXT LEVEL,' a six-month sponsorship and leadership development program partnered with employee resource groups to build a diverse leadership bench | FY26 Impact Report cites a third cohort of a six-month global leadership development experience with 20 employees combining sponsorship, skill-building, and applied learning on real business challenges</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Workday 10-K human capital section summaries; workday.com Career Hub pages</t>
+          <t>Autodesk News TLDP/NEXT LEVEL articles; Autodesk FY25/FY26 Impact Report</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Autodesk, Inc.</t>
+          <t>Adobe Inc.</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1714,31 +1719,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C41" s="1" t="inlineStr">
-        <is>
-          <t>https://www.autodesk.com</t>
-        </is>
-      </c>
-      <c r="D41" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/769397/000076939726000015/adsk-20260131.htm</t>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://www.adobe.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/796343/000079634326000003/adbe-20251128.htm</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Ran a six-month Tech Lead Development Program (TLDP) cohort for rising non-technical leaders, with 66% of participants promoted or given new responsibilities during/after the program and 88% saying it helped drive success for their organization | Runs 'NEXT LEVEL,' a six-month sponsorship and leadership development program partnered with employee resource groups to build a diverse leadership bench | FY26 Impact Report cites a third cohort of a six-month global leadership development experience with 20 employees combining sponsorship, skill-building, and applied learning on real business challenges</t>
+          <t>Adobe's Learning Fund reimburses employees up to $10,000/year for undergraduate, graduate, PhD, MBA degrees and select professional certifications | Separate Professional Development Reimbursement covers up to $1,000/year for conferences, webinars, online courses, and professional memberships | Adobe Digital University learning platform has reached 42,000+ employees, customers and partners with structured digital-skills courses</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Autodesk News TLDP/NEXT LEVEL articles; Autodesk FY25/FY26 Impact Report</t>
+          <t>Adobe FY2025 10-K (SEC); benefits.adobe.com; Adobe Digital University case study</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Adobe Inc.</t>
+          <t>Intuit Inc.</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1746,31 +1751,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C42" s="1" t="inlineStr">
-        <is>
-          <t>https://www.adobe.com</t>
-        </is>
-      </c>
-      <c r="D42" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/796343/000079634326000003/adbe-20251128.htm</t>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://www.intuit.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/896878/000089687825000035/intu-20250731.htm</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Adobe's Learning Fund reimburses employees up to $10,000/year for undergraduate, graduate, PhD, MBA degrees and select professional certifications | Separate Professional Development Reimbursement covers up to $1,000/year for conferences, webinars, online courses, and professional memberships | Adobe Digital University learning platform has reached 42,000+ employees, customers and partners with structured digital-skills courses</t>
+          <t>Intuit's FY2025 10-K describes company-sponsored learning paths and online courses spanning topics from AI to 'accelerating velocity,' available to all full-time employees | Named internal program 'Intuit Leadership Playbook' targets manager and executive leadership-skill development | Learning is structured across the employee lifecycle starting at onboarding, paired with an internal-mobility focus to help employees acquire new skills and take on new roles</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Adobe FY2025 10-K (SEC); benefits.adobe.com; Adobe Digital University case study</t>
+          <t>Intuit Inc. FY2025 Form 10-K, Human Capital section (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Intuit Inc.</t>
+          <t>Citrix Systems, Inc.</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1778,31 +1783,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C43" s="1" t="inlineStr">
-        <is>
-          <t>https://www.intuit.com</t>
-        </is>
-      </c>
-      <c r="D43" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/896878/000089687825000035/intu-20250731.htm</t>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://www.citrix.com</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Intuit's FY2025 10-K describes company-sponsored learning paths and online courses spanning topics from AI to 'accelerating velocity,' available to all full-time employees | Named internal program 'Intuit Leadership Playbook' targets manager and executive leadership-skill development | Learning is structured across the employee lifecycle starting at onboarding, paired with an internal-mobility focus to help employees acquire new skills and take on new roles</t>
+          <t>as a public company (pre-2022 privatization), Citrix's 10-K human capital section referenced mentoring/coaching programs and a large library of on-demand learning resources for its ~9,700 employees, but disclosed no specific training-hour or dollar figures | Citrix Education's external certification tracks suggest an internal culture already oriented toward structured technical certification, plausibly extended to staff upskilling | given heavy IT/virtualization focus, internal L&amp;D probably emphasized technical re-certification and product training over broad tuition-reimbursement programs</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Intuit Inc. FY2025 Form 10-K, Human Capital section (SEC EDGAR)</t>
+          <t>Citrix Systems FY2021 Form 10-K human capital disclosure; Citrix Education public pages â€” no specific metrics found post-2022 privatization</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Citrix Systems, Inc.</t>
+          <t>Symantec Corporation</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1810,26 +1810,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C44" s="1" t="inlineStr">
-        <is>
-          <t>https://www.citrix.com</t>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://www.symantec.com</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>as a public company (pre-2022 privatization), Citrix's 10-K human capital section referenced mentoring/coaching programs and a large library of on-demand learning resources for its ~9,700 employees, but disclosed no specific training-hour or dollar figures | Citrix Education's external certification tracks suggest an internal culture already oriented toward structured technical certification, plausibly extended to staff upskilling | given heavy IT/virtualization focus, internal L&amp;D probably emphasized technical re-certification and product training over broad tuition-reimbursement programs</t>
+          <t>pre-acquisition Symantec (last full-year filer ~FY2018) was reported to offer tuition reimbursement for work-related degrees/certificates alongside coaching and mentoring programs | as a large cybersecurity vendor, Symantec plausibly ran onboarding and technical-certification training to keep staff current on its own security product certifications | no specific training-hour, dollar-investment, or named-program figures could be confirmed from the FY2018 10-K's human capital disclosures before the Broadcom enterprise-security acquisition</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Citrix Systems FY2021 Form 10-K human capital disclosure; Citrix Education public pages â€” no specific metrics found post-2022 privatization</t>
+          <t>Secondary benefits summary referencing Symantec tuition reimbursement/mentoring; Symantec FY2018 10-K</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Symantec Corporation</t>
+          <t>Zscaler, Inc.</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1837,26 +1837,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C45" s="1" t="inlineStr">
-        <is>
-          <t>https://www.symantec.com</t>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://www.zscaler.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1713683/000171368325000158/zs-20250731.htm</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>pre-acquisition Symantec (last full-year filer ~FY2018) was reported to offer tuition reimbursement for work-related degrees/certificates alongside coaching and mentoring programs | as a large cybersecurity vendor, Symantec plausibly ran onboarding and technical-certification training to keep staff current on its own security product certifications | no specific training-hour, dollar-investment, or named-program figures could be confirmed from the FY2018 10-K's human capital disclosures before the Broadcom enterprise-security acquisition</t>
+          <t>Zscaler's FY2025 10-K states new Customer Care/Success hires go through structured sales and product training programs | Technical teams get live and online training resources plus frequent internal 'tech talks' on best practices and product developments | Company offers tuition reimbursement for eligible employees pursuing higher education, plus external-expert-led leadership development for senior leaders</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Secondary benefits summary referencing Symantec tuition reimbursement/mentoring; Symantec FY2018 10-K</t>
+          <t>Zscaler, Inc. FY2025 Form 10-K, Human Capital section (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Zscaler, Inc.</t>
+          <t>RingCentral, Inc.</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1864,31 +1869,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C46" s="1" t="inlineStr">
-        <is>
-          <t>https://www.zscaler.com</t>
-        </is>
-      </c>
-      <c r="D46" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1713683/000171368325000158/zs-20250731.htm</t>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.ringcentral.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1384905/000138490526000021/rng-20251231.htm</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Zscaler's FY2025 10-K states new Customer Care/Success hires go through structured sales and product training programs | Technical teams get live and online training resources plus frequent internal 'tech talks' on best practices and product developments | Company offers tuition reimbursement for eligible employees pursuing higher education, plus external-expert-led leadership development for senior leaders</t>
+          <t>Learning courses offered across leadership, inclusion and diversity, technical and compliance categories | Company runs structured talent development programs aimed at helping employees grow in current roles and build new skills | Has won external awards recognizing its leadership development and onboarding programs</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Zscaler, Inc. FY2025 Form 10-K, Human Capital section (SEC EDGAR)</t>
+          <t>RingCentral FY2025 10-K (SEC) human capital section</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>RingCentral, Inc.</t>
+          <t>ZoomInfo Technologies, Inc.</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1896,31 +1901,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C47" s="1" t="inlineStr">
-        <is>
-          <t>https://www.ringcentral.com</t>
-        </is>
-      </c>
-      <c r="D47" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1384905/000138490526000021/rng-20251231.htm</t>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://www.zoominfo.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=ZI</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Learning courses offered across leadership, inclusion and diversity, technical and compliance categories | Company runs structured talent development programs aimed at helping employees grow in current roles and build new skills | Has won external awards recognizing its leadership development and onboarding programs</t>
+          <t>Invests in 'robust learning offerings' combining online courses and live training for all employees, with targeted tracks for individual contributors vs. leaders | Global Inclusion and Diversity Initiative (GIDI) ties professional development and diversity education together as a formal program | 3,508 employees as of FY2024 covered by these development practices</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>RingCentral FY2025 10-K (SEC) human capital section</t>
+          <t>ZoomInfo Technologies FY2024 10-K (SEC) human capital section</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ZoomInfo Technologies, Inc.</t>
+          <t>Five9, Inc.</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1928,31 +1933,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C48" s="1" t="inlineStr">
-        <is>
-          <t>https://www.zoominfo.com</t>
-        </is>
-      </c>
-      <c r="D48" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=ZI</t>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://www.five9.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1288847/000128884726000023/fivn-20251231.htm</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Invests in 'robust learning offerings' combining online courses and live training for all employees, with targeted tracks for individual contributors vs. leaders | Global Inclusion and Diversity Initiative (GIDI) ties professional development and diversity education together as a formal program | 3,508 employees as of FY2024 covered by these development practices</t>
+          <t>Talent development built around company Leadership Principles that guide Talent Acquisition, Learning and Development, and Performance Management practices | Formal mentor-mentee pairing program run by HR to give employees structured growth opportunities | 2,684 full-time employees as of FY2023; company also hires dedicated Learning Program Manager roles for GTM enablement</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>ZoomInfo Technologies FY2024 10-K (SEC) human capital section</t>
+          <t>Five9 10-K filings (SEC); Five9 careers listings</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Five9, Inc.</t>
+          <t>Bill.com Holdings, Inc.</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1960,31 +1965,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C49" s="1" t="inlineStr">
-        <is>
-          <t>https://www.five9.com</t>
-        </is>
-      </c>
-      <c r="D49" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1288847/000128884726000023/fivn-20251231.htm</t>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://www.bill.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1786352/000178635225000037/bill-20250630.htm</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Talent development built around company Leadership Principles that guide Talent Acquisition, Learning and Development, and Performance Management practices | Formal mentor-mentee pairing program run by HR to give employees structured growth opportunities | 2,684 full-time employees as of FY2023; company also hires dedicated Learning Program Manager roles for GTM enablement</t>
+          <t>Cohort-based 'key talent' leadership programs plus mandatory training for new people managers | Employees get access to an online learning curriculum via a third-party platform tied to business needs; launched a 2025 'Summer of AI' initiative teaching staff to use internal AI tools | Runs a quarterly Leadership Speaker Series with internal/external subject-matter experts, alongside twice-yearly performance review cycles</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Five9 10-K filings (SEC); Five9 careers listings</t>
+          <t>BILL Holdings FY2025 10-K (SEC) human capital section</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Bill.com Holdings, Inc.</t>
+          <t>SentinelOne, Inc.</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1992,31 +1997,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C50" s="1" t="inlineStr">
-        <is>
-          <t>https://www.bill.com</t>
-        </is>
-      </c>
-      <c r="D50" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1786352/000178635225000037/bill-20250630.htm</t>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.sentinelone.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1583708/000158370826000020/s-20260131.htm</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Cohort-based 'key talent' leadership programs plus mandatory training for new people managers | Employees get access to an online learning curriculum via a third-party platform tied to business needs; launched a 2025 'Summer of AI' initiative teaching staff to use internal AI tools | Runs a quarterly Leadership Speaker Series with internal/external subject-matter experts, alongside twice-yearly performance review cycles</t>
+          <t>Built a role-based learning strategy with an external partner, creating structured learning pathways by level rather than one-size-fits-all training | Co-launched a company-wide GenAI training cohort in 2024 combining AI workshops, AMA sessions, and Slack-based peer knowledge sharing | Runs 'SentinelOne University,' a public-facing cybersecurity training/certification arm, alongside a WiCyS apprenticeship partnership for underrepresented talent</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>BILL Holdings FY2025 10-K (SEC) human capital section</t>
+          <t>SentinelOne FY2026 10-K (SEC) human capital section</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SentinelOne, Inc.</t>
+          <t>Cyberark Software Ltd.</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2024,31 +2029,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C51" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sentinelone.com</t>
-        </is>
-      </c>
-      <c r="D51" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1583708/000158370826000020/s-20260131.htm</t>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://www.cyberark.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=CYBR</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Built a role-based learning strategy with an external partner, creating structured learning pathways by level rather than one-size-fits-all training | Co-launched a company-wide GenAI training cohort in 2024 combining AI workshops, AMA sessions, and Slack-based peer knowledge sharing | Runs 'SentinelOne University,' a public-facing cybersecurity training/certification arm, alongside a WiCyS apprenticeship partnership for underrepresented talent</t>
+          <t>CyberArk's Chief Human Resources Officer reports directly to the CEO and leads a human capital management strategy focused on developing and retaining top diverse talent | Company runs frequent mandatory training on Code of Conduct, anti-corruption, insider trading, data privacy and cybersecurity as part of a three-pillar ethics/compliance program | New Board members receive tailored onboarding training and ongoing director education via internally developed materials</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>SentinelOne FY2026 10-K (SEC) human capital section</t>
+          <t>CyberArk Software Ltd. 20-F/6-K filings (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Cyberark Software Ltd.</t>
+          <t>Ping Identity Holding Corp.</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2056,31 +2061,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C52" s="1" t="inlineStr">
-        <is>
-          <t>https://www.cyberark.com</t>
-        </is>
-      </c>
-      <c r="D52" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=CYBR</t>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://www.pingidentity.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=PING</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>CyberArk's Chief Human Resources Officer reports directly to the CEO and leads a human capital management strategy focused on developing and retaining top diverse talent | Company runs frequent mandatory training on Code of Conduct, anti-corruption, insider trading, data privacy and cybersecurity as part of a three-pillar ethics/compliance program | New Board members receive tailored onboarding training and ongoing director education via internally developed materials</t>
+          <t>As a technical identity-security vendor, Ping Identity's engineering and support staff likely required continuous training to stay current across multiple deployment environments per its last 10-K (FY2021) | Total rewards program suggests investment in broader employee development and retention prior to its 2022 Thoma Bravo take-private | Company conducted periodic pay equity analyses via independent third parties, indicating a structured people-development/HR governance process</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>CyberArk Software Ltd. 20-F/6-K filings (SEC EDGAR)</t>
+          <t>Ping Identity Holding Corp. FY2021 10-K â€” company went private in 2022, no filings since</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ping Identity Holding Corp.</t>
+          <t>Qualys, Inc.</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2088,31 +2093,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C53" s="1" t="inlineStr">
-        <is>
-          <t>https://www.pingidentity.com</t>
-        </is>
-      </c>
-      <c r="D53" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=PING</t>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://www.qualys.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1107843/000110784326000008/qlys-20251231.htm</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>As a technical identity-security vendor, Ping Identity's engineering and support staff likely required continuous training to stay current across multiple deployment environments per its last 10-K (FY2021) | Total rewards program suggests investment in broader employee development and retention prior to its 2022 Thoma Bravo take-private | Company conducted periodic pay equity analyses via independent third parties, indicating a structured people-development/HR governance process</t>
+          <t>Qualys offers free self-paced and instructor-led certified training on core Qualys product topics, letting employees earn certifications and job-related courses at no cost | All new hires complete a structured onboarding program tailored to role-specific functions and company culture | Formal annual employee performance reviews plus regular HR-manager check-ins support ongoing career development, alongside mandatory harassment-prevention/diversity/security training</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Ping Identity Holding Corp. FY2021 10-K â€” company went private in 2022, no filings since</t>
+          <t>Qualys, Inc. FY2025 10-K (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Qualys, Inc.</t>
+          <t>Rapid7, Inc.</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2120,31 +2125,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C54" s="1" t="inlineStr">
-        <is>
-          <t>https://www.qualys.com</t>
-        </is>
-      </c>
-      <c r="D54" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1107843/000110784326000008/qlys-20251231.htm</t>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://www.rapid7.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1560327/000156032726000008/rp-20251231.htm</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Qualys offers free self-paced and instructor-led certified training on core Qualys product topics, letting employees earn certifications and job-related courses at no cost | All new hires complete a structured onboarding program tailored to role-specific functions and company culture | Formal annual employee performance reviews plus regular HR-manager check-ins support ongoing career development, alongside mandatory harassment-prevention/diversity/security training</t>
+          <t>Rapid7's human capital strategy emphasizes building a 'dynamic and collaborative workplace' with multidimensional teams and programs supporting employee wellbeing to help staff 'build fulfilling careers' | As of FY2025, Rapid7 had 2,613 full-time employees globally, a scale that typically requires structured onboarding and role-based technical training for security-product staff | No collective bargaining coverage in the U.S. and company reports good employee relations, consistent with internally managed HR/development programs</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Qualys, Inc. FY2025 10-K (SEC EDGAR)</t>
+          <t>Rapid7, Inc. FY2025 10-K (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Rapid7, Inc.</t>
+          <t>SailPoint Technologies Holdings, Inc.</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2152,31 +2157,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C55" s="1" t="inlineStr">
-        <is>
-          <t>https://www.rapid7.com</t>
-        </is>
-      </c>
-      <c r="D55" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1560327/000156032726000008/rp-20251231.htm</t>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://www.sailpoint.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/2030781/000203078126000003/sail-20260131.htm</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Rapid7's human capital strategy emphasizes building a 'dynamic and collaborative workplace' with multidimensional teams and programs supporting employee wellbeing to help staff 'build fulfilling careers' | As of FY2025, Rapid7 had 2,613 full-time employees globally, a scale that typically requires structured onboarding and role-based technical training for security-product staff | No collective bargaining coverage in the U.S. and company reports good employee relations, consistent with internally managed HR/development programs</t>
+          <t>SailPoint's human capital strategy explicitly names 'career development and training opportunities' as a core pillar alongside team-member engagement to attract and retain talent | Leaders undergo specific training to embed company core values into team management decisions | Diversity/inclusion training targets bias removal from recruiting, paired with pay equity reviews during merit planning; overall team-member satisfaction held at 90% for four consecutive survey years</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Rapid7, Inc. FY2025 10-K (SEC EDGAR)</t>
+          <t>SailPoint Technologies Holdings, Inc. 10-K filings (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SailPoint Technologies Holdings, Inc.</t>
+          <t>Varonis Systems, Inc.</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2184,31 +2189,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C56" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sailpoint.com</t>
-        </is>
-      </c>
-      <c r="D56" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/2030781/000203078126000003/sail-20260131.htm</t>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://www.varonis.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1361113/000162828026005450/vrns-20251231.htm</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SailPoint's human capital strategy explicitly names 'career development and training opportunities' as a core pillar alongside team-member engagement to attract and retain talent | Leaders undergo specific training to embed company core values into team management decisions | Diversity/inclusion training targets bias removal from recruiting, paired with pay equity reviews during merit planning; overall team-member satisfaction held at 90% for four consecutive survey years</t>
+          <t>UpSkill Academy gives all employees access to live, interactive sessions on communication, time management, prioritization, growth mindset, and feedback | New managers complete a 12-week nomination-based program to build people-leadership skills, plus two-day workshops for managers at all levels | Internal mobility program helps employees explore career paths across departments, alongside on-demand learning and professional certification resources</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>SailPoint Technologies Holdings, Inc. 10-K filings (SEC EDGAR)</t>
+          <t>Varonis careers page; Varonis 10-K FY2025 (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Varonis Systems, Inc.</t>
+          <t>NetApp, Inc.</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2216,31 +2221,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C57" s="1" t="inlineStr">
-        <is>
-          <t>https://www.varonis.com</t>
-        </is>
-      </c>
-      <c r="D57" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1361113/000162828026005450/vrns-20251231.htm</t>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://www.netapp.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1002047/000119312526259683/ntap-20260424.htm</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>UpSkill Academy gives all employees access to live, interactive sessions on communication, time management, prioritization, growth mindset, and feedback | New managers complete a 12-week nomination-based program to build people-leadership skills, plus two-day workshops for managers at all levels | Internal mobility program helps employees explore career paths across departments, alongside on-demand learning and professional certification resources</t>
+          <t>Educational assistance/tuition reimbursement program reported to provide up to $5,000 per calendar year for job-related coursework | Growth goals are tied to corporate OKRs, with managers conducting quarterly two-way career-development conversations | Offers online and classroom-based learning including courses, certifications, webinars, and formal mentorship programs; Talent and Compensation Committee of the Board oversees talent/development strategy</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Varonis careers page; Varonis 10-K FY2025 (SEC EDGAR)</t>
+          <t>NetApp 10-K filings (SEC EDGAR); Glassdoor/third-party benefit summaries</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>NetApp, Inc.</t>
+          <t>Pure Storage, Inc.</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2248,31 +2253,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C58" s="1" t="inlineStr">
-        <is>
-          <t>https://www.netapp.com</t>
-        </is>
-      </c>
-      <c r="D58" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1002047/000119312526259683/ntap-20260424.htm</t>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://www.purestorage.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=PSTG</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Educational assistance/tuition reimbursement program reported to provide up to $5,000 per calendar year for job-related coursework | Growth goals are tied to corporate OKRs, with managers conducting quarterly two-way career-development conversations | Offers online and classroom-based learning including courses, certifications, webinars, and formal mentorship programs; Talent and Compensation Committee of the Board oversees talent/development strategy</t>
+          <t>10-K human capital disclosure states the company provides training and development programs so employees can build products/services that further career goals and corporate mission | Runs global performance management and internal mobility programs to support employee growth | Deploys a third-party 'Pulse of Pure' engagement survey measuring career development, manager effectiveness, and inclusion, with leaders reviewing results quarterly</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>NetApp 10-K filings (SEC EDGAR); Glassdoor/third-party benefit summaries</t>
+          <t>Pure Storage Form 10-K (SEC EDGAR, FY2025)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Pure Storage, Inc.</t>
+          <t>Nutanix, Inc.</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2280,31 +2285,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C59" s="1" t="inlineStr">
-        <is>
-          <t>https://www.purestorage.com</t>
-        </is>
-      </c>
-      <c r="D59" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=PSTG</t>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://www.nutanix.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1618732/000119312525213801/ntnx-20250731.htm</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>10-K human capital disclosure states the company provides training and development programs so employees can build products/services that further career goals and corporate mission | Runs global performance management and internal mobility programs to support employee growth | Deploys a third-party 'Pulse of Pure' engagement survey measuring career development, manager effectiveness, and inclusion, with leaders reviewing results quarterly</t>
+          <t>10-K states the company invests significant resources to foster a learning culture and empower employees' personal/professional growth via extensive onboarding and training programs | Learning programs include digital learning, speed coaching, customized workshops, and management-enablement/skills training for current, new, and future managers | Also runs DEI training and language-learning programs; ~7,800 employees worldwide as of July 31, 2025</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Pure Storage Form 10-K (SEC EDGAR, FY2025)</t>
+          <t>Nutanix Form 10-K (SEC EDGAR, FY2025)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Nutanix, Inc.</t>
+          <t>Analog Devices, Inc.</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2312,31 +2317,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C60" s="1" t="inlineStr">
-        <is>
-          <t>https://www.nutanix.com</t>
-        </is>
-      </c>
-      <c r="D60" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1618732/000119312525213801/ntnx-20250731.htm</t>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://www.analog.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/6281/000000628125000153/adi-20251101.htm</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>10-K states the company invests significant resources to foster a learning culture and empower employees' personal/professional growth via extensive onboarding and training programs | Learning programs include digital learning, speed coaching, customized workshops, and management-enablement/skills training for current, new, and future managers | Also runs DEI training and language-learning programs; ~7,800 employees worldwide as of July 31, 2025</t>
+          <t>Offers employee education through the ADI Academy brand, providing flexible, expert-led learning with curated learning paths | 10-K human capital section cites employee surveys used to gauge effectiveness of development and compensation programs | FY2024 voluntary employee turnover was approximately 8%, cited alongside retention/development objectives</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Nutanix Form 10-K (SEC EDGAR, FY2025)</t>
+          <t>Analog Devices Form 10-K (SEC EDGAR); ADI Academy (ez.analog.com/adiacademy)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Analog Devices, Inc.</t>
+          <t>ON Semiconductor Corporation</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2344,31 +2349,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C61" s="1" t="inlineStr">
-        <is>
-          <t>https://www.analog.com</t>
-        </is>
-      </c>
-      <c r="D61" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/6281/000000628125000153/adi-20251101.htm</t>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://www.onsemi.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1097864/000109786426000006/on-20251231.htm</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Offers employee education through the ADI Academy brand, providing flexible, expert-led learning with curated learning paths | 10-K human capital section cites employee surveys used to gauge effectiveness of development and compensation programs | FY2024 voluntary employee turnover was approximately 8%, cited alongside retention/development objectives</t>
+          <t>onsemi 2025 Employee Engagement Survey had 95% employee participation | ON Semiconductor Foundation awarded $1.35M to 37 organizations in 2025 for STEAM/tech-skills education | Company earned MSCI ESG 'A' rating for 7 consecutive years (through Oct 2025), tied partly to workforce development practices</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Analog Devices Form 10-K (SEC EDGAR); ADI Academy (ez.analog.com/adiacademy)</t>
+          <t>onsemi 2024/2025 Sustainability Report</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ON Semiconductor Corporation</t>
+          <t>KLA Corporation</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2376,31 +2381,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C62" s="1" t="inlineStr">
-        <is>
-          <t>https://www.onsemi.com</t>
-        </is>
-      </c>
-      <c r="D62" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1097864/000109786426000006/on-20251231.htm</t>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://www.kla.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/319201/000031920125000024/klac-20250630.htm</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>onsemi 2025 Employee Engagement Survey had 95% employee participation | ON Semiconductor Foundation awarded $1.35M to 37 organizations in 2025 for STEAM/tech-skills education | Company earned MSCI ESG 'A' rating for 7 consecutive years (through Oct 2025), tied partly to workforce development practices</t>
+          <t>KLA offers tuition reimbursement plus custom advanced-engineering-degree partnerships with Stanford University and University of Michigan | New customer/technical service engineers complete up to 12 weeks of onsite, hands-on product training before field deployment | Formal coaching/mentorship program and performance process built around frequent 1:1 manager coaching and feedback</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>onsemi 2024/2025 Sustainability Report</t>
+          <t>KLA FY2025 10-K human capital section; kla.com/advance/education</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>KLA Corporation</t>
+          <t>Lam Research Corporation</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2408,31 +2413,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C63" s="1" t="inlineStr">
-        <is>
-          <t>https://www.kla.com</t>
-        </is>
-      </c>
-      <c r="D63" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/319201/000031920125000024/klac-20250630.htm</t>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://www.lamresearch.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/707549/000070754925000075/lrcx-20250629.htm</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>KLA offers tuition reimbursement plus custom advanced-engineering-degree partnerships with Stanford University and University of Michigan | New customer/technical service engineers complete up to 12 weeks of onsite, hands-on product training before field deployment | Formal coaching/mentorship program and performance process built around frequent 1:1 manager coaching and feedback</t>
+          <t>Lam Research logged 480,000 training hours across 3,042 distinct courses in a recent reporting year | Runs structured mentorship, coaching, and job-rotation programs to accelerate employee career development | People managers in field support, manufacturing, R&amp;D, warehouse and logistics undergo formal safety leadership training biannually</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>KLA FY2025 10-K human capital section; kla.com/advance/education</t>
+          <t>Lam Research 10-K human capital disclosures; Lam CSR Report</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Lam Research Corporation</t>
+          <t>Applied Materials, Inc.</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2440,31 +2445,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C64" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lamresearch.com</t>
-        </is>
-      </c>
-      <c r="D64" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/707549/000070754925000075/lrcx-20250629.htm</t>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://www.appliedmaterials.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/6951/000162828025056742/amat-20251026.htm</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Lam Research logged 480,000 training hours across 3,042 distinct courses in a recent reporting year | Runs structured mentorship, coaching, and job-rotation programs to accelerate employee career development | People managers in field support, manufacturing, R&amp;D, warehouse and logistics undergo formal safety leadership training biannually</t>
+          <t>Applied Materials requires every employee to complete 40 hours of learning per fiscal year, supplemented by university coursework and professional accreditation | Historically over 85% of employees carry a formal individual development goal as part of performance objectives | Runs Applied Global Services 'Academy' programs (recognized as a Training Top 125 best practice) targeting functional skill-building teams</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Lam Research 10-K human capital disclosures; Lam CSR Report</t>
+          <t>Applied Materials Learning &amp; Development addendum; Training magazine Top 125</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Applied Materials, Inc.</t>
+          <t>Cadence Design Systems, Inc.</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2472,31 +2477,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C65" s="1" t="inlineStr">
-        <is>
-          <t>https://www.appliedmaterials.com</t>
-        </is>
-      </c>
-      <c r="D65" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/6951/000162828025056742/amat-20251026.htm</t>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://www.cadence.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/813672/000081367226000016/cdns-20251231.htm</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Applied Materials requires every employee to complete 40 hours of learning per fiscal year, supplemented by university coursework and professional accreditation | Historically over 85% of employees carry a formal individual development goal as part of performance objectives | Runs Applied Global Services 'Academy' programs (recognized as a Training Top 125 best practice) targeting functional skill-building teams</t>
+          <t>Cadence provides a comprehensive online Learning Management System covering a broad range of technical and professional topics, plus formal training curricula and on-the-job training | Offers tuition reimbursement to employees pursuing further education | Leaders are formally measured on talent attraction, development, and engagement as part of the company's 'One Team' human capital strategy</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Applied Materials Learning &amp; Development addendum; Training magazine Top 125</t>
+          <t>Cadence Design Systems FY2025 10-K human capital section</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Cadence Design Systems, Inc.</t>
+          <t>Synopsys, Inc.</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2504,31 +2509,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C66" s="1" t="inlineStr">
-        <is>
-          <t>https://www.cadence.com</t>
-        </is>
-      </c>
-      <c r="D66" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/813672/000081367226000016/cdns-20251231.htm</t>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://www.synopsys.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/883241/000088324125000028/snps-20251031.htm</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Cadence provides a comprehensive online Learning Management System covering a broad range of technical and professional topics, plus formal training curricula and on-the-job training | Offers tuition reimbursement to employees pursuing further education | Leaders are formally measured on talent attraction, development, and engagement as part of the company's 'One Team' human capital strategy</t>
+          <t>People strategy built on five pillars including 'Foster Learning and Growth' and 'Accelerate Next Gen Synopsys' | ~28,000 employees company-wide, ~75% engineers, over half with Master's or PhD degrees | Runs Synopsys Learning Center offering self-paced training, badging, and certification programs for technical skill development</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Cadence Design Systems FY2025 10-K human capital section</t>
+          <t>Synopsys FY2025 10-K human capital section</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Synopsys, Inc.</t>
+          <t>Akamai Technologies, Inc.</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2536,31 +2541,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C67" s="1" t="inlineStr">
-        <is>
-          <t>https://www.synopsys.com</t>
-        </is>
-      </c>
-      <c r="D67" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/883241/000088324125000028/snps-20251031.htm</t>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://www.akamai.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1086222/000108622226000022/akam-20251231.htm</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>People strategy built on five pillars including 'Foster Learning and Growth' and 'Accelerate Next Gen Synopsys' | ~28,000 employees company-wide, ~75% engineers, over half with Master's or PhD degrees | Runs Synopsys Learning Center offering self-paced training, badging, and certification programs for technical skill development</t>
+          <t>Akamai University provides global technical training and certifications, including the Akamai Certified DevOps Associate (ACDA) curriculum for solutions architects and delivery leads | Akamai Technical Academy (ATA) trains non-traditional-background hires with foundational technical and soft-skills training for entry-level tech roles | Employee benefits include tuition assistance alongside mentoring, leadership development programs, and cross-functional project rotations</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Synopsys FY2025 10-K human capital section</t>
+          <t>Akamai FY2023-2025 10-K human capital disclosures</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Akamai Technologies, Inc.</t>
+          <t>Arista Networks, Inc.</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2568,31 +2573,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C68" s="1" t="inlineStr">
-        <is>
-          <t>https://www.akamai.com</t>
-        </is>
-      </c>
-      <c r="D68" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1086222/000108622226000022/akam-20251231.htm</t>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://www.arista.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1596532/000159653226000013/anet-20251231.htm</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Akamai University provides global technical training and certifications, including the Akamai Certified DevOps Associate (ACDA) curriculum for solutions architects and delivery leads | Akamai Technical Academy (ATA) trains non-traditional-background hires with foundational technical and soft-skills training for entry-level tech roles | Employee benefits include tuition assistance alongside mentoring, leadership development programs, and cross-functional project rotations</t>
+          <t>Arista Certified Engineering (ACE) certification/accreditation program covers Sales, Customer Engineering, and Software R&amp;D employees | Internal 'Arista PREP Training Program' plus technical summits and industry conference participation support technical employee upskilling | E-Learning portal offers management and AI training content, and mandatory periodic training on ethics, infosec, data privacy, IP, and anticorruption</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Akamai FY2023-2025 10-K human capital disclosures</t>
+          <t>Arista Networks FY2024 10-K human capital section</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Arista Networks, Inc.</t>
+          <t>ASGN Incorporated</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2600,31 +2605,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C69" s="1" t="inlineStr">
-        <is>
-          <t>https://www.arista.com</t>
-        </is>
-      </c>
-      <c r="D69" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1596532/000159653226000013/anet-20251231.htm</t>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://www.asgn.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=ASGN</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Arista Certified Engineering (ACE) certification/accreditation program covers Sales, Customer Engineering, and Software R&amp;D employees | Internal 'Arista PREP Training Program' plus technical summits and industry conference participation support technical employee upskilling | E-Learning portal offers management and AI training content, and mandatory periodic training on ethics, infosec, data privacy, IP, and anticorruption</t>
+          <t>as an IT/engineering staffing and consulting firm, ASGN likely reimburses or subsidizes technical certifications (cloud, cybersecurity, PMP-type credentials) to keep consultants billable and current | internal L&amp;D probably centers on onboarding and role-specific upskilling for recruiters, delivery leads, and technical consultants rather than a large formal corporate academy | certification and continuing-education support is likely positioned as a client-facing credibility requirement rather than a broad-based employee development program</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Arista Networks FY2024 10-K human capital section</t>
+          <t>ASGN human capital messaging â€” no concrete 10-K figures found</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ASGN Incorporated</t>
+          <t>Box, Inc.</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2632,31 +2637,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C70" s="1" t="inlineStr">
-        <is>
-          <t>https://www.asgn.com</t>
-        </is>
-      </c>
-      <c r="D70" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=ASGN</t>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://www.box.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1372612/000119312526098466/box-20260131.htm</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>as an IT/engineering staffing and consulting firm, ASGN likely reimburses or subsidizes technical certifications (cloud, cybersecurity, PMP-type credentials) to keep consultants billable and current | internal L&amp;D probably centers on onboarding and role-specific upskilling for recruiters, delivery leads, and technical consultants rather than a large formal corporate academy | certification and continuing-education support is likely positioned as a client-facing credibility requirement rather than a broad-based employee development program</t>
+          <t>Runs 'LearnFest,' a twice-yearly company-wide learning event with trainings, workshops, and book clubs for skill development | Provides director-level-and-above employees access to executive programs including Harvard's Leadership Consortium and Stanford's Women's Executive Leadership programs | On-demand learning platform offers 2,000+ courses, including 600+ on personal development, management, and leadership plus hundreds of technical/functional skill courses</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>ASGN human capital messaging â€” no concrete 10-K figures found</t>
+          <t>Box, Inc. 10-K human capital disclosures</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Box, Inc.</t>
+          <t>Check Point Software Technologies Ltd.</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2664,31 +2669,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C71" s="1" t="inlineStr">
-        <is>
-          <t>https://www.box.com</t>
-        </is>
-      </c>
-      <c r="D71" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1372612/000119312526098466/box-20260131.htm</t>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://www.checkpoint.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=CHKP</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Runs 'LearnFest,' a twice-yearly company-wide learning event with trainings, workshops, and book clubs for skill development | Provides director-level-and-above employees access to executive programs including Harvard's Leadership Consortium and Stanford's Women's Executive Leadership programs | On-demand learning platform offers 2,000+ courses, including 600+ on personal development, management, and leadership plus hundreds of technical/functional skill courses</t>
+          <t>Runs UniverCP, an internal Learning Management System offering self-paced online training 24/7 on technical skills, soft skills, Check Point solutions, tools/processes, and managerial best practices | Maintains a formal Training and Employee Development Policy plus entry-level onboarding and instructor-led courses for new hires | Also runs an external Training &amp; Certification business via its own academy, Coursera, and edX, reflecting a strong internal certification culture</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Box, Inc. 10-K human capital disclosures</t>
+          <t>Check Point corporate site; ESG Training and Employee Development Policy</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Check Point Software Technologies Ltd.</t>
+          <t>Ciena Corporation</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2696,31 +2701,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C72" s="1" t="inlineStr">
-        <is>
-          <t>https://www.checkpoint.com</t>
-        </is>
-      </c>
-      <c r="D72" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=CHKP</t>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://www.ciena.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/936395/000162828025056698/cien-20251101.htm</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Runs UniverCP, an internal Learning Management System offering self-paced online training 24/7 on technical skills, soft skills, Check Point solutions, tools/processes, and managerial best practices | Maintains a formal Training and Employee Development Policy plus entry-level onboarding and instructor-led courses for new hires | Also runs an external Training &amp; Certification business via its own academy, Coursera, and edX, reflecting a strong internal certification culture</t>
+          <t>Human capital strategy centers on recruiting, developing, and retaining talent, with ~8,657 employees and investment in people development framed as a core corporate strategy pillar | Offers early-in-career/new graduate programs, management and leadership development programs, coaching/mentoring, and tuition reimbursement for continuing education | Runs mandatory Code of Business Conduct and Ethics training with recurring affirmations, plus a formal leadership succession planning process</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Check Point corporate site; ESG Training and Employee Development Policy</t>
+          <t>Ciena FY2024 10-K human capital section</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Ciena Corporation</t>
+          <t>Commvault Systems, Inc.</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2728,31 +2733,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C73" s="1" t="inlineStr">
-        <is>
-          <t>https://www.ciena.com</t>
-        </is>
-      </c>
-      <c r="D73" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/936395/000162828025056698/cien-20251101.htm</t>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://www.commvault.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1169561/000116956126000017/cvlt-20260331.htm</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Human capital strategy centers on recruiting, developing, and retaining talent, with ~8,657 employees and investment in people development framed as a core corporate strategy pillar | Offers early-in-career/new graduate programs, management and leadership development programs, coaching/mentoring, and tuition reimbursement for continuing education | Runs mandatory Code of Business Conduct and Ethics training with recurring affirmations, plus a formal leadership succession planning process</t>
+          <t>In fiscal 2025, employees, partners, and customers participated in over 1,400 training programs totaling more than 260,000 hours (up from 1,200+ programs / 190,000+ hours in FY2024) | Fiscal 2026 saw launch of new mandatory cybersecurity and AI governance training programs for all employees, with 3,400+ training programs totaling 219,000+ hours company-wide | ~3,300 employees worldwide, with Employee Resource Groups and DEI-linked professional development initiatives</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Ciena FY2024 10-K human capital section</t>
+          <t>Commvault FY2024-FY2026 10-K human capital disclosures</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Commvault Systems, Inc.</t>
+          <t>Cornerstone OnDemand, Inc.</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2760,31 +2765,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C74" s="1" t="inlineStr">
-        <is>
-          <t>https://www.commvault.com</t>
-        </is>
-      </c>
-      <c r="D74" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1169561/000116956126000017/cvlt-20260331.htm</t>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://www.cornerstoneondemand.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=CSOD</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>In fiscal 2025, employees, partners, and customers participated in over 1,400 training programs totaling more than 260,000 hours (up from 1,200+ programs / 190,000+ hours in FY2024) | Fiscal 2026 saw launch of new mandatory cybersecurity and AI governance training programs for all employees, with 3,400+ training programs totaling 219,000+ hours company-wide | ~3,300 employees worldwide, with Employee Resource Groups and DEI-linked professional development initiatives</t>
+          <t>Runs quarterly global 'Development Days,' internally organized by employees for professional and personal development classes | Culture built around continuous personal growth, with company self-reporting 85% of employees rating it a great place to work vs 57% industry average | As an L&amp;D/talent-management software vendor itself (now private under Clearlake Capital since 2021), the company's own product (Cornerstone learning platform) is used internally to run its training and development programs</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Commvault FY2024-FY2026 10-K human capital disclosures</t>
+          <t>cornerstoneondemand.com/careers; Great Place to Work certification page</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand, Inc.</t>
+          <t>CyberCore Technologies</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2792,31 +2797,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C75" s="1" t="inlineStr">
-        <is>
-          <t>https://www.cornerstoneondemand.com</t>
-        </is>
-      </c>
-      <c r="D75" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=CSOD</t>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://www.cybercoretech.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=CYBR</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Runs quarterly global 'Development Days,' internally organized by employees for professional and personal development classes | Culture built around continuous personal growth, with company self-reporting 85% of employees rating it a great place to work vs 57% industry average | As an L&amp;D/talent-management software vendor itself (now private under Clearlake Capital since 2021), the company's own product (Cornerstone learning platform) is used internally to run its training and development programs</t>
+          <t>Operates a formal career development program called 'Compass' pairing each employee with a dedicated career development specialist | Provides continuing education benefits of up to $10,000 per employee for education/training, unlimited training time, and free access to online IT courses, plus an on-site training lab/sandbox for hands-on tool practice | Offers a certification incentive program and training reimbursement, aimed at security-cleared IT/defense professionals maintaining industry certifications</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>cornerstoneondemand.com/careers; Great Place to Work certification page</t>
+          <t>cybercoretech.com careers pages</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CyberCore Technologies</t>
+          <t>DigitalOcean Holdings, Inc.</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2824,31 +2829,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C76" s="1" t="inlineStr">
-        <is>
-          <t>https://www.cybercoretech.com</t>
-        </is>
-      </c>
-      <c r="D76" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=CYBR</t>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://www.digitalocean.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1582961/000158296126000019/docn-20251231.htm</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Operates a formal career development program called 'Compass' pairing each employee with a dedicated career development specialist | Provides continuing education benefits of up to $10,000 per employee for education/training, unlimited training time, and free access to online IT courses, plus an on-site training lab/sandbox for hands-on tool practice | Offers a certification incentive program and training reimbursement, aimed at security-cleared IT/defense professionals maintaining industry certifications</t>
+          <t>Employees get unlimited access to LinkedIn Learning plus a monthly book-purchase benefit ('Book Program') for professional growth | New engineers go through a structured 4-6 week onboarding covering DigitalOcean's tech stack (Go, Python, React) and internal tools | Career development includes personalized learning budgets, internal tech talks/workshops, mentorship pairing junior with senior staff, and defined promotion pathways</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>cybercoretech.com careers pages</t>
+          <t>DigitalOcean careers/People Team pages; FY2025 10-K human capital section</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>DigitalOcean Holdings, Inc.</t>
+          <t>Domo, Inc.</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2856,31 +2861,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C77" s="1" t="inlineStr">
-        <is>
-          <t>https://www.digitalocean.com</t>
-        </is>
-      </c>
-      <c r="D77" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1582961/000158296126000019/docn-20251231.htm</t>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://www.domo.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1505952/000162828026025356/domo-20260131.htm</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Employees get unlimited access to LinkedIn Learning plus a monthly book-purchase benefit ('Book Program') for professional growth | New engineers go through a structured 4-6 week onboarding covering DigitalOcean's tech stack (Go, Python, React) and internal tools | Career development includes personalized learning budgets, internal tech talks/workshops, mentorship pairing junior with senior staff, and defined promotion pathways</t>
+          <t>Runs 'Domo University,' a self-paced and instructor-led training/certification program originally built for customers but reflecting the company's broader learning infrastructure | Domo employees rate 'career opportunities' 3.2/5 and comp/benefits 3.7/5 on Glassdoor, with reviewers citing internal promotion of execs as evidence of upward mobility | offers standard SaaS-company benefits bundle but no publicly disclosed specific employee training budget, hours, or named internal L&amp;D program was found</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>DigitalOcean careers/People Team pages; FY2025 10-K human capital section</t>
+          <t>Domo.com (Domo University); Glassdoor company reviews/benefits pages</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Domo, Inc.</t>
+          <t>Ellucian Company L.P.</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2888,31 +2893,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C78" s="1" t="inlineStr">
-        <is>
-          <t>https://www.domo.com</t>
-        </is>
-      </c>
-      <c r="D78" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1505952/000162828026025356/domo-20260131.htm</t>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://www.ellucian.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=ELUC</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Runs 'Domo University,' a self-paced and instructor-led training/certification program originally built for customers but reflecting the company's broader learning infrastructure | Domo employees rate 'career opportunities' 3.2/5 and comp/benefits 3.7/5 on Glassdoor, with reviewers citing internal promotion of execs as evidence of upward mobility | offers standard SaaS-company benefits bundle but no publicly disclosed specific employee training budget, hours, or named internal L&amp;D program was found</t>
+          <t>Runs a formal Learning &amp; Development team offering workshops, training platforms and mentorship, plus tuition reimbursement for approved courses/degrees for all full-time employees | Named programs include a 12-month 'Immersive Onboarding Experience,' a Leadership Development track, quarterly 'TalentFest' professional development conference, and 'Ellucian Academy' for upskilling/reskilling | Company has 4,000+ employees and emphasizes daily interactive exercises to embed skill development into day-to-day work</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Domo.com (Domo University); Glassdoor company reviews/benefits pages</t>
+          <t>Ellucian careers/values-in-action pages</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Ellucian Company L.P.</t>
+          <t>F5, Inc.</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2920,31 +2925,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C79" s="1" t="inlineStr">
-        <is>
-          <t>https://www.ellucian.com</t>
-        </is>
-      </c>
-      <c r="D79" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=ELUC</t>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://www.f5.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1048695/000104869525000157/ffiv-20250930.htm</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Runs a formal Learning &amp; Development team offering workshops, training platforms and mentorship, plus tuition reimbursement for approved courses/degrees for all full-time employees | Named programs include a 12-month 'Immersive Onboarding Experience,' a Leadership Development track, quarterly 'TalentFest' professional development conference, and 'Ellucian Academy' for upskilling/reskilling | Company has 4,000+ employees and emphasizes daily interactive exercises to embed skill development into day-to-day work</t>
+          <t>FY2025 10-K human capital section states F5 invested in tailored coaching and skills-building for people managers, delivered via live events (Innovation Months, Idea Fests, Technology Days, Learning Days) | Offers tuition assistance for professional development and a comprehensive global mentoring/sponsorship program alongside leadership coaching | Maintains 7 Employee Inclusion Groups (active since 2013) that also serve as peer learning communities</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Ellucian careers/values-in-action pages</t>
+          <t>F5 Inc FY2025 10-K human capital section</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>F5, Inc.</t>
+          <t>FireEye, Inc.</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2952,31 +2957,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C80" s="1" t="inlineStr">
-        <is>
-          <t>https://www.f5.com</t>
-        </is>
-      </c>
-      <c r="D80" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1048695/000104869525000157/ffiv-20250930.htm</t>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://www.fireeye.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=FEYE</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>FY2025 10-K human capital section states F5 invested in tailored coaching and skills-building for people managers, delivered via live events (Innovation Months, Idea Fests, Technology Days, Learning Days) | Offers tuition assistance for professional development and a comprehensive global mentoring/sponsorship program alongside leadership coaching | Maintains 7 Employee Inclusion Groups (active since 2013) that also serve as peer learning communities</t>
+          <t>FireEye no longer exists as a standalone company: its products business merged with McAfee Enterprise in Jan 2022 to form Trellix, while Mandiant was carved out and sold to Google Cloud in 2022 | Under Google, 'Mandiant Academy' continues running paid instructor-led and online security training/certification courses for customers | as Trellix/Mandiant are now owned by private equity (STG) and Google respectively, internal employee L&amp;D likely follows each parent's standard corporate training and certification-support programs rather than any surviving 'FireEye' program</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>F5 Inc FY2025 10-K human capital section</t>
+          <t>CyberScoop, Wikipedia (Trellix), Google Cloud Mandiant Academy course listings</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>FireEye, Inc.</t>
+          <t>Fortinet, Inc.</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2984,31 +2989,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C81" s="1" t="inlineStr">
-        <is>
-          <t>https://www.fireeye.com</t>
-        </is>
-      </c>
-      <c r="D81" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=FEYE</t>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://www.fortinet.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1262039/000126203926000007/ftnt-20251231.htm</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>FireEye no longer exists as a standalone company: its products business merged with McAfee Enterprise in Jan 2022 to form Trellix, while Mandiant was carved out and sold to Google Cloud in 2022 | Under Google, 'Mandiant Academy' continues running paid instructor-led and online security training/certification courses for customers | as Trellix/Mandiant are now owned by private equity (STG) and Google respectively, internal employee L&amp;D likely follows each parent's standard corporate training and certification-support programs rather than any surviving 'FireEye' program</t>
+          <t>Fortinet Training Institute has issued approximately 2 million certifications to date, covering employees, customers, partners, and the public | Employees get free access to Fortinet's own security training programs (NSE certification tracks) for career development | Fortinet Training Institute partners with industry, academia, government, and nonprofits worldwide to close the cybersecurity skills gap, with an internal training team building curriculum alongside technical experts</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>CyberScoop, Wikipedia (Trellix), Google Cloud Mandiant Academy course listings</t>
+          <t>Fortinet FY2025 10-K Human Capital section</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Fortinet, Inc.</t>
+          <t>Guidewire Software, Inc.</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3016,31 +3021,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C82" s="1" t="inlineStr">
-        <is>
-          <t>https://www.fortinet.com</t>
-        </is>
-      </c>
-      <c r="D82" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1262039/000126203926000007/ftnt-20251231.htm</t>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://www.guidewire.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1528396/000152839625000221/gwre-20250731.htm</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Fortinet Training Institute has issued approximately 2 million certifications to date, covering employees, customers, partners, and the public | Employees get free access to Fortinet's own security training programs (NSE certification tracks) for career development | Fortinet Training Institute partners with industry, academia, government, and nonprofits worldwide to close the cybersecurity skills gap, with an internal training team building curriculum alongside technical experts</t>
+          <t>Guidewire invests in broad-based employee development including cutting-edge skills training, on-demand AI learning platforms, and dynamic mentorship programs | Company runs transformative leadership development programs alongside regular professional education to support career progression | Guidewire tracks L&amp;D effectiveness via annual talent reviews, employee feedback, and promotion/hiring goal data across its ~3,772 employees</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Fortinet FY2025 10-K Human Capital section</t>
+          <t>Guidewire FY2025 10-K Human Capital Management section</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Guidewire Software, Inc.</t>
+          <t>HashiCorp, Inc.</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3048,31 +3053,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C83" s="1" t="inlineStr">
-        <is>
-          <t>https://www.guidewire.com</t>
-        </is>
-      </c>
-      <c r="D83" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1528396/000152839625000221/gwre-20250731.htm</t>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://www.hashicorp.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=HCP</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Guidewire invests in broad-based employee development including cutting-edge skills training, on-demand AI learning platforms, and dynamic mentorship programs | Company runs transformative leadership development programs alongside regular professional education to support career progression | Guidewire tracks L&amp;D effectiveness via annual talent reviews, employee feedback, and promotion/hiring goal data across its ~3,772 employees</t>
+          <t>Prior to its Feb 2025 acquisition by IBM, HashiCorp described investment in talent development, manager enablement, and knowledge-sharing programs to support employee career growth | HashiCorp ran an Early Careers/internship program that included structured onboarding and development events for junior talent | Post-acquisition, HashiCorp employees have gained access to IBM's broader enterprise learning and R&amp;D career-development infrastructure</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Guidewire FY2025 10-K Human Capital Management section</t>
+          <t>HashiCorp careers site and company blog â€” no standalone 10-K exists for FY2025+</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>HashiCorp, Inc.</t>
+          <t>Informatica Inc.</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3080,31 +3085,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C84" s="1" t="inlineStr">
-        <is>
-          <t>https://www.hashicorp.com</t>
-        </is>
-      </c>
-      <c r="D84" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=HCP</t>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://www.informatica.com</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=INFA</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Prior to its Feb 2025 acquisition by IBM, HashiCorp described investment in talent development, manager enablement, and knowledge-sharing programs to support employee career growth | HashiCorp ran an Early Careers/internship program that included structured onboarding and development events for junior talent | Post-acquisition, HashiCorp employees have gained access to IBM's broader enterprise learning and R&amp;D career-development infrastructure</t>
+          <t>Informatica University offers structured Training Paths (1-3 classes plus a certification) mapped to specific product roles, available live or virtually for employees and customers | Company offers a tuition reimbursement benefit of up to $5,250/year for job-related coursework, requiring a grade of B- or better | FY2024 10-K Human Capital section (5,200+ full-time employees) cites employee-driven recognition programs and regular feedback surveys used to shape workplace/development initiatives</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>HashiCorp careers site and company blog â€” no standalone 10-K exists for FY2025+</t>
+          <t>Informatica FY2024 10-K Human Capital Management section</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Informatica Inc.</t>
+          <t>JFrog Ltd.</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3112,31 +3117,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C85" s="1" t="inlineStr">
-        <is>
-          <t>https://www.informatica.com</t>
-        </is>
-      </c>
-      <c r="D85" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=INFA</t>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://www.jfrog.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1800667/000119312526051382/frog-20251231.htm</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Informatica University offers structured Training Paths (1-3 classes plus a certification) mapped to specific product roles, available live or virtually for employees and customers | Company offers a tuition reimbursement benefit of up to $5,250/year for job-related coursework, requiring a grade of B- or better | FY2024 10-K Human Capital section (5,200+ full-time employees) cites employee-driven recognition programs and regular feedback surveys used to shape workplace/development initiatives</t>
+          <t>JFrog runs formal and informal cross-company training programs specifically to prepare new managers and employees for career growth within the company | JFrog Academy offers free self-paced courses plus paid instructor-led training, with Associate-level certifications in JFrog Artifactory and JFrog Security | All ~1,800 JFrog employees receive mandatory security-awareness and privacy-awareness training at onboarding plus mandatory annual refreshers</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Informatica FY2024 10-K Human Capital Management section</t>
+          <t>JFrog FY2025 10-K Human Capital Management section</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>JFrog Ltd.</t>
+          <t>Juniper Networks, Inc.</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -3144,31 +3149,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C86" s="1" t="inlineStr">
-        <is>
-          <t>https://www.jfrog.com</t>
-        </is>
-      </c>
-      <c r="D86" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1800667/000119312526051382/frog-20251231.htm</t>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://www.juniper.net</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=JNPR</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>JFrog runs formal and informal cross-company training programs specifically to prepare new managers and employees for career growth within the company | JFrog Academy offers free self-paced courses plus paid instructor-led training, with Associate-level certifications in JFrog Artifactory and JFrog Security | All ~1,800 JFrog employees receive mandatory security-awareness and privacy-awareness training at onboarding plus mandatory annual refreshers</t>
+          <t>Launched Junivator Career Connect (JCC) in 2023, an internal talent marketplace for customized learning journeys, mentor connections, and internal gig work | Provides company-wide LinkedIn Learning access covering business, technology, and creative skills courses | Uses 'Talent Matters' framework for annual role-specific compliance and development training plus manager-led growth assessments (last available as standalone filer pre-HPE acquisition)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>JFrog FY2025 10-K Human Capital Management section</t>
+          <t>Juniper Networks 10-K filings (SEC EDGAR) and 2017-18 Corporate Citizenship &amp; Sustainability Report</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Juniper Networks, Inc.</t>
+          <t>Mellanox Technologies, Ltd.</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3176,31 +3181,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C87" s="1" t="inlineStr">
-        <is>
-          <t>https://www.juniper.net</t>
-        </is>
-      </c>
-      <c r="D87" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=JNPR</t>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://www.mellanox.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=MLNX</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Launched Junivator Career Connect (JCC) in 2023, an internal talent marketplace for customized learning journeys, mentor connections, and internal gig work | Provides company-wide LinkedIn Learning access covering business, technology, and creative skills courses | Uses 'Talent Matters' framework for annual role-specific compliance and development training plus manager-led growth assessments (last available as standalone filer pre-HPE acquisition)</t>
+          <t>Mellanox employees were absorbed into NVIDIA's human capital programs after the 2020 acquisition, including NVIDIA's tuition reimbursement for degrees and professional certifications | NVIDIA runs a career coaching service plus mentoring/peer-coaching programs and a library of live/on-demand workshops and learning paths for all staff including ex-Mellanox teams | NVIDIA's Deep Learning Institute (DLI), while primarily external-facing, is also used internally for technical upskilling of engineering staff</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Juniper Networks 10-K filings (SEC EDGAR) and 2017-18 Corporate Citizenship &amp; Sustainability Report</t>
+          <t>NVIDIA 10-K (SEC EDGAR) and NVIDIA Corporate Responsibility Reports</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Mellanox Technologies, Ltd.</t>
+          <t>Micro Focus International plc</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -3208,31 +3213,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C88" s="1" t="inlineStr">
-        <is>
-          <t>https://www.mellanox.com</t>
-        </is>
-      </c>
-      <c r="D88" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=MLNX</t>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://www.microfocus.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=MFGP</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Mellanox employees were absorbed into NVIDIA's human capital programs after the 2020 acquisition, including NVIDIA's tuition reimbursement for degrees and professional certifications | NVIDIA runs a career coaching service plus mentoring/peer-coaching programs and a library of live/on-demand workshops and learning paths for all staff including ex-Mellanox teams | NVIDIA's Deep Learning Institute (DLI), while primarily external-facing, is also used internally for technical upskilling of engineering staff</t>
+          <t>Micro Focus's training/L&amp;D programs are now folded into OpenText's after the 2023 acquisition, run under OpenText's 'Zero-In' ESG framework | OpenText offers education/tuition reimbursement plus formal leadership and management training tracks for people managers | All OpenText managers complete a mandatory 'Hiring the Best' course (incl. unconscious-bias training) and a 'Leading a Diverse Workforce' course</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>NVIDIA 10-K (SEC EDGAR) and NVIDIA Corporate Responsibility Reports</t>
+          <t>OpenText Corporate Citizenship Reports</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Micro Focus International plc</t>
+          <t>MongoDB, Inc.</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3240,31 +3245,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C89" s="1" t="inlineStr">
-        <is>
-          <t>https://www.microfocus.com</t>
-        </is>
-      </c>
-      <c r="D89" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=MFGP</t>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://www.mongodb.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1441816/000162828026016799/mdb-20260131.htm</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Micro Focus's training/L&amp;D programs are now folded into OpenText's after the 2023 acquisition, run under OpenText's 'Zero-In' ESG framework | OpenText offers education/tuition reimbursement plus formal leadership and management training tracks for people managers | All OpenText managers complete a mandatory 'Hiring the Best' course (incl. unconscious-bias training) and a 'Leading a Diverse Workforce' course</t>
+          <t>Development happens largely on-the-job as the company scales, with frequent role expansion giving employees stretch opportunities | Runs a formal 'performance and growth framework' with continuous manager feedback plus semi-annual performance/growth conversations and individual development plans | Leadership development is delivered via structured and customized programming for managers at every level, anchored in MongoDB's own documented Leadership Principles</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>OpenText Corporate Citizenship Reports</t>
+          <t>MongoDB, Inc. FY2026 Form 10-K (SEC EDGAR), Human Capital section</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>MongoDB, Inc.</t>
+          <t>NCR Corporation</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3272,31 +3277,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C90" s="1" t="inlineStr">
-        <is>
-          <t>https://www.mongodb.com</t>
-        </is>
-      </c>
-      <c r="D90" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1441816/000162828026016799/mdb-20260131.htm</t>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://www.ncr.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=NCR</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Development happens largely on-the-job as the company scales, with frequent role expansion giving employees stretch opportunities | Runs a formal 'performance and growth framework' with continuous manager feedback plus semi-annual performance/growth conversations and individual development plans | Leadership development is delivered via structured and customized programming for managers at every level, anchored in MongoDB's own documented Leadership Principles</t>
+          <t>Runs 'NCR Voyix University,' an internal online education platform for continuous employee learning, and partners with external L&amp;D platforms to uplevel global workforce capabilities | Offers a tuition assistance program covering college and graduate-level programs tied to business-critical skills | Board's Risk Committee provides direct oversight of ESG programs covering people development and DEI, across roughly 15,500 employees worldwide</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>MongoDB, Inc. FY2026 Form 10-K (SEC EDGAR), Human Capital section</t>
+          <t>NCR Voyix Corp FY2023 Form 10-K (SEC EDGAR), Human Capital Management section</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>NCR Corporation</t>
+          <t>Palo Alto Networks, Inc.</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -3304,31 +3309,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C91" s="1" t="inlineStr">
-        <is>
-          <t>https://www.ncr.com</t>
-        </is>
-      </c>
-      <c r="D91" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=NCR</t>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://www.paloaltonetworks.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000027/panw-20250731.htm</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Runs 'NCR Voyix University,' an internal online education platform for continuous employee learning, and partners with external L&amp;D platforms to uplevel global workforce capabilities | Offers a tuition assistance program covering college and graduate-level programs tied to business-critical skills | Board's Risk Committee provides direct oversight of ESG programs covering people development and DEI, across roughly 15,500 employees worldwide</t>
+          <t>Learning and enablement is one of four core pillars of Palo Alto Networks' People Strategy, overseen by the Chief People Officer with regular board updates | FY2025 10-K describes active integration of AI into people programs to build a more agile, skilled, forward-thinking workforce for cybersecurity roles | Recruitment and internal skills strategy prioritizes durable 'AI-readiness' capabilities given rapid technical skill evolution, across a 16,068-person global workforce</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>NCR Voyix Corp FY2023 Form 10-K (SEC EDGAR), Human Capital Management section</t>
+          <t>Palo Alto Networks FY2025 10-K (SEC), Human Capital section</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Palo Alto Networks, Inc.</t>
+          <t>Paycom Software, Inc.</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -3336,31 +3341,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C92" s="1" t="inlineStr">
-        <is>
-          <t>https://www.paloaltonetworks.com</t>
-        </is>
-      </c>
-      <c r="D92" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000027/panw-20250731.htm</t>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://www.paycom.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1590955/000119312526059372/payc-20251231.htm</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Learning and enablement is one of four core pillars of Palo Alto Networks' People Strategy, overseen by the Chief People Officer with regular board updates | FY2025 10-K describes active integration of AI into people programs to build a more agile, skilled, forward-thinking workforce for cybersecurity roles | Recruitment and internal skills strategy prioritizes durable 'AI-readiness' capabilities given rapid technical skill evolution, across a 16,068-person global workforce</t>
+          <t>Paycom Learning (proprietary LMS) delivers self-guided, tailored learning paths in leadership, DEI, technical skills and compliance; in 2020 employees completed thousands of unique courses through the tool | Sales organization completes a structured 10-week onboarding/training course before taking on client accounts, cited as a top-rated sales training program | PIX/L, an internal IT conference, plus on-site coaching from dedicated development coaches support ongoing career growth (3x consecutive Comparably 'Best Career Growth' award winner through 2024) across a 5,770-employee base</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Palo Alto Networks FY2025 10-K (SEC), Human Capital section</t>
+          <t>Paycom 10-K filings (SEC EDGAR) FY2020/FY2025 Human Capital sections</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Paycom Software, Inc.</t>
+          <t>Pegasystems Inc.</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3368,31 +3373,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C93" s="1" t="inlineStr">
-        <is>
-          <t>https://www.paycom.com</t>
-        </is>
-      </c>
-      <c r="D93" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1590955/000119312526059372/payc-20251231.htm</t>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://www.pega.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1013857/000101385726000017/pega-20251231.htm</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Paycom Learning (proprietary LMS) delivers self-guided, tailored learning paths in leadership, DEI, technical skills and compliance; in 2020 employees completed thousands of unique courses through the tool | Sales organization completes a structured 10-week onboarding/training course before taking on client accounts, cited as a top-rated sales training program | PIX/L, an internal IT conference, plus on-site coaching from dedicated development coaches support ongoing career growth (3x consecutive Comparably 'Best Career Growth' award winner through 2024) across a 5,770-employee base</t>
+          <t>Pega Academy is a named internal platform giving employees (plus clients/partners) structured Pega software skills training and certification paths | Five distinct cohort-based leadership development programs target people managers and leaders across all functions and geographies, alongside education reimbursement programs | 10-K human capital disclosures state over 90% of employees participated in a formal education program and frame 'lifelong learning' as a core company philosophy</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Paycom 10-K filings (SEC EDGAR) FY2020/FY2025 Human Capital sections</t>
+          <t>Pegasystems 10-K filings (SEC EDGAR), FY2020 and FY2025 Human Capital sections</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Pegasystems Inc.</t>
+          <t>Proofpoint, Inc.</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -3400,31 +3405,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C94" s="1" t="inlineStr">
-        <is>
-          <t>https://www.pega.com</t>
-        </is>
-      </c>
-      <c r="D94" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1013857/000101385726000017/pega-20251231.htm</t>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://www.proofpoint.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=PFPT</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Pega Academy is a named internal platform giving employees (plus clients/partners) structured Pega software skills training and certification paths | Five distinct cohort-based leadership development programs target people managers and leaders across all functions and geographies, alongside education reimbursement programs | 10-K human capital disclosures state over 90% of employees participated in a formal education program and frame 'lifelong learning' as a core company philosophy</t>
+          <t>Elevate is Proofpoint's named leadership-development program focused on building modern leadership skills and personal growth for people managers | Employees get access to internal security-awareness training content plus support toward industry certifications such as CISSP and CEH, alongside skills courses on time-management, delegation, and crucial conversations | Since 2021 Thoma Bravo take-private, no public 10-K/ESG disclosures exist; L&amp;D detail now sourced only from proofpoint.com corporate-responsibility page</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Pegasystems 10-K filings (SEC EDGAR), FY2020 and FY2025 Human Capital sections</t>
+          <t>proofpoint.com/us/legal/corporate-responsibility/talent-development â€” post-2021 private company, no SEC filings</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Proofpoint, Inc.</t>
+          <t>RealPage, Inc.</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -3432,31 +3437,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C95" s="1" t="inlineStr">
-        <is>
-          <t>https://www.proofpoint.com</t>
-        </is>
-      </c>
-      <c r="D95" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=PFPT</t>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://www.realpage.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=RP</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Elevate is Proofpoint's named leadership-development program focused on building modern leadership skills and personal growth for people managers | Employees get access to internal security-awareness training content plus support toward industry certifications such as CISSP and CEH, alongside skills courses on time-management, delegation, and crucial conversations | Since 2021 Thoma Bravo take-private, no public 10-K/ESG disclosures exist; L&amp;D detail now sourced only from proofpoint.com corporate-responsibility page</t>
+          <t>RealConnect is RealPage's named LMS, used both for customer/product training and internally to build role-based 'learning pathways' by position, market type, and location | Company offers a structured tuition reimbursement program plus access to external learning content (e.g., LinkedIn Learning) alongside internal courses | Since 2021 Thoma Bravo take-private, no public 10-K/ESG filings exist; certified a 'Great Place to Work' in the US, UK, India, Philippines and Colombia</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>proofpoint.com/us/legal/corporate-responsibility/talent-development â€” post-2021 private company, no SEC filings</t>
+          <t>realpage.com training/LMS pages; Glassdoor/Indeed employee reviews â€” post-2021 private company, no SEC filings</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>RealPage, Inc.</t>
+          <t>Roper Technologies, Inc.</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3464,31 +3469,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C96" s="1" t="inlineStr">
-        <is>
-          <t>https://www.realpage.com</t>
-        </is>
-      </c>
-      <c r="D96" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=RP</t>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://www.ropertech.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/882835/000088283526000009/rop-20251231.htm</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>RealConnect is RealPage's named LMS, used both for customer/product training and internally to build role-based 'learning pathways' by position, market type, and location | Company offers a structured tuition reimbursement program plus access to external learning content (e.g., LinkedIn Learning) alongside internal courses | Since 2021 Thoma Bravo take-private, no public 10-K/ESG filings exist; certified a 'Great Place to Work' in the US, UK, India, Philippines and Colombia</t>
+          <t>Roper's decentralized operating model puts human capital decisions, including leadership development and succession planning, in the hands of individual business unit managers rather than a centralized L&amp;D function | Corporate HQ shares best practices across ~19,400 employees on talent selection, development, engagement and excellence | Investing in leadership development and succession planning is explicitly named a key human capital priority in the FY2025 10-K</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>realpage.com training/LMS pages; Glassdoor/Indeed employee reviews â€” post-2021 private company, no SEC filings</t>
+          <t>Roper Technologies FY2025 10-K (SEC EDGAR), Human Capital section</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Roper Technologies, Inc.</t>
+          <t>Sangamo Therapeutics, Inc.</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3496,31 +3501,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C97" s="1" t="inlineStr">
-        <is>
-          <t>https://www.ropertech.com</t>
-        </is>
-      </c>
-      <c r="D97" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/882835/000088283526000009/rop-20251231.htm</t>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://www.sangamo.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1001233/000162828026022029/sgmo-20251231.htm</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Roper's decentralized operating model puts human capital decisions, including leadership development and succession planning, in the hands of individual business unit managers rather than a centralized L&amp;D function | Corporate HQ shares best practices across ~19,400 employees on talent selection, development, engagement and excellence | Investing in leadership development and succession planning is explicitly named a key human capital priority in the FY2025 10-K</t>
+          <t>as a clinical-stage genomic medicine biotech, Sangamo likely relies on informal mentoring and role-specific scientific/GxP training rather than a named corporate university or large-scale program | given its small headcount, professional development is probably individualized (conference attendance, certifications relevant to genomic medicine/regulatory affairs) rather than disclosed with hard metrics | DEF 14A proxy and careers page emphasize culture and employee growth qualitatively but do not appear to publish training hours, spend, or named program figures</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Roper Technologies FY2025 10-K (SEC EDGAR), Human Capital section</t>
+          <t>Sangamo careers page and SEC DEF 14A search â€” no quantified training disclosures found</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Sangamo Therapeutics, Inc.</t>
+          <t>SecureWorks Corp.</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3528,31 +3533,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C98" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sangamo.com</t>
-        </is>
-      </c>
-      <c r="D98" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1001233/000162828026022029/sgmo-20251231.htm</t>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://www.secureworks.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=SCWX</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>as a clinical-stage genomic medicine biotech, Sangamo likely relies on informal mentoring and role-specific scientific/GxP training rather than a named corporate university or large-scale program | given its small headcount, professional development is probably individualized (conference attendance, certifications relevant to genomic medicine/regulatory affairs) rather than disclosed with hard metrics | DEF 14A proxy and careers page emphasize culture and employee growth qualitatively but do not appear to publish training hours, spend, or named program figures</t>
+          <t>Secureworks was taken private by Sophos in 2025, ending separate public ESG/10-K disclosure of its training programs | Parent Sophos runs a formal L&amp;D program offering three paid learning days (24 hours) per employee per year for workshops, coaching, mentoring, or self-paced learning | Sophos also runs an Internal Coaching Scheme and a structured early-career mentorship program with two six-month cohorts annually</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Sangamo careers page and SEC DEF 14A search â€” no quantified training disclosures found</t>
+          <t>Sophos careers/L&amp;D page; Secureworks now a Sophos subsidiary post-2025 acquisition</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SecureWorks Corp.</t>
+          <t>SiTime Corporation</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3560,31 +3565,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C99" s="1" t="inlineStr">
-        <is>
-          <t>https://www.secureworks.com</t>
-        </is>
-      </c>
-      <c r="D99" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=SCWX</t>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://www.sitime.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1451809/000145180926000012/sitm-20251231.htm</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Secureworks was taken private by Sophos in 2025, ending separate public ESG/10-K disclosure of its training programs | Parent Sophos runs a formal L&amp;D program offering three paid learning days (24 hours) per employee per year for workshops, coaching, mentoring, or self-paced learning | Sophos also runs an Internal Coaching Scheme and a structured early-career mentorship program with two six-month cohorts annually</t>
+          <t>SiTime's FY2025 10-K human capital section states the company 'encourages all employees to continue learning' and provides cross-functional internal mobility opportunities to support development | Managers and employees hold periodic structured conversations covering feedback, goal alignment, and professional development plans | All employees receive mandatory annual training on cybersecurity awareness and protection of confidential information, alongside ongoing succession planning to promote internal talent</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Sophos careers/L&amp;D page; Secureworks now a Sophos subsidiary post-2025 acquisition</t>
+          <t>SiTime Corporation 10-K (SEC EDGAR), Human Capital Resources section</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SiTime Corporation</t>
+          <t>Skyworks Solutions, Inc.</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3592,259 +3597,28 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C100" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sitime.com</t>
-        </is>
-      </c>
-      <c r="D100" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1451809/000145180926000012/sitm-20251231.htm</t>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://www.skyworksinc.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/4127/000000412725000085/swks-20251003.htm</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>SiTime's FY2025 10-K human capital section states the company 'encourages all employees to continue learning' and provides cross-functional internal mobility opportunities to support development | Managers and employees hold periodic structured conversations covering feedback, goal alignment, and professional development plans | All employees receive mandatory annual training on cybersecurity awareness and protection of confidential information, alongside ongoing succession planning to promote internal talent</t>
+          <t>Skyworks offers tuition reimbursement covering up to 25% of costs for team members pursuing a job-related certificate or degree, plus partial reimbursement (25%) toward GED completion | Educational assistance is bundled under an internally branded 'Invest in the Future' benefits category alongside learning/development and recognition programs | New hires go through a structured onboarding program designed to integrate them into teams and ongoing projects</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>SiTime Corporation 10-K (SEC EDGAR), Human Capital Resources section</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>Skyworks Solutions, Inc.</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C101" s="1" t="inlineStr">
-        <is>
-          <t>https://www.skyworksinc.com</t>
-        </is>
-      </c>
-      <c r="D101" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/4127/000000412725000085/swks-20251003.htm</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>Skyworks offers tuition reimbursement covering up to 25% of costs for team members pursuing a job-related certificate or degree, plus partial reimbursement (25%) toward GED completion | Educational assistance is bundled under an internally branded 'Invest in the Future' benefits category alongside learning/development and recognition programs | New hires go through a structured onboarding program designed to integrate them into teams and ongoing projects</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
           <t>Skyworks Solutions benefits disclosures (Levels.fyi/Glassdoor benefits pages)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId197"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>